<commit_message>
BL : catalogue au format du registre (Z:BB), N° de ligne + N° de série, réf catalogue reprise
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XPwnZBmWUGhvYebrP3X3Z2
</commit_message>
<xml_diff>
--- a/bl_2027/BL_Enedril_2027.xlsx
+++ b/bl_2027/BL_Enedril_2027.xlsx
@@ -168,7 +168,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -215,6 +215,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="002E8B57"/>
         <bgColor rgb="002E8B57"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F5F9"/>
+        <bgColor rgb="00F2F5F9"/>
       </patternFill>
     </fill>
   </fills>
@@ -332,7 +338,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -469,6 +475,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -893,7 +902,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O69"/>
+  <dimension ref="A1:P69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -909,8 +918,9 @@
     <col hidden="1" width="13" customWidth="1" min="11" max="11"/>
     <col hidden="1" width="13" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
     <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -1063,8 +1073,8 @@
     <row r="14" ht="36" customHeight="1">
       <c r="A14" s="12" t="inlineStr">
         <is>
-          <t>Réf
-Ref</t>
+          <t>N°
+Item</t>
         </is>
       </c>
       <c r="B14" s="12" t="inlineStr">
@@ -1109,15 +1119,20 @@
       </c>
       <c r="M14" s="14" t="inlineStr">
         <is>
+          <t>Réf catalogue</t>
+        </is>
+      </c>
+      <c r="N14" s="14" t="inlineStr">
+        <is>
           <t>Code SH</t>
         </is>
       </c>
-      <c r="N14" s="14" t="inlineStr">
+      <c r="O14" s="14" t="inlineStr">
         <is>
           <t>OD</t>
         </is>
       </c>
-      <c r="O14" s="14" t="inlineStr">
+      <c r="P14" s="14" t="inlineStr">
         <is>
           <t>Lg</t>
         </is>
@@ -1125,12 +1140,12 @@
     </row>
     <row r="15" ht="26" customHeight="1">
       <c r="A15" s="15">
-        <f>IF(L15&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L15),"")</f>
+        <f>IF(OR(J15=0,K15=1),"",COUNTIF(K$15:K15,0)-COUNTIF(J$15:J15,0))</f>
         <v/>
       </c>
       <c r="B15" s="15" t="n"/>
       <c r="C15" s="16">
-        <f>IF(J15=0,"",IF(K15=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J15)),IF(L15&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L15),INDEX('2 Import devis'!$B$6:$B$29,J15))))</f>
+        <f>IF(J15=0,"",IF(K15=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J15)),IF(L15&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L15,2)),INDEX('2 Import devis'!$B$6:$B$29,J15))))</f>
         <v/>
       </c>
       <c r="D15" s="17">
@@ -1138,11 +1153,11 @@
         <v/>
       </c>
       <c r="E15" s="17">
-        <f>IF(K15=1,"",IF(L15&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L15)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L15)),"FR"))</f>
+        <f>IF(OR(J15=0,K15=1),"",IF(L15&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L15,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L15,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L15,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F15" s="18">
-        <f>IF(L15&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L15)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L15)),"")</f>
+        <f>IF(L15&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L15,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L15,3),1)),"")</f>
         <v/>
       </c>
       <c r="G15" s="19">
@@ -1166,26 +1181,30 @@
         <v/>
       </c>
       <c r="M15" s="20">
-        <f>IF(L15&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L15)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L15)),"")</f>
+        <f>IF(L15&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L15,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L15,20)),"")</f>
         <v/>
       </c>
       <c r="N15" s="20">
-        <f>IF(L15&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L15)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L15)),"")</f>
+        <f>IF(L15&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L15,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L15,23)),"")</f>
         <v/>
       </c>
       <c r="O15" s="20">
-        <f>IF(L15&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L15)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L15)),"")</f>
+        <f>IF(L15&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L15,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L15,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P15" s="20">
+        <f>IF(L15&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L15,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L15,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="16" ht="26" customHeight="1">
       <c r="A16" s="15">
-        <f>IF(L16&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L16),"")</f>
+        <f>IF(OR(J16=0,K16=1),"",COUNTIF(K$15:K16,0)-COUNTIF(J$15:J16,0))</f>
         <v/>
       </c>
       <c r="B16" s="15" t="n"/>
       <c r="C16" s="16">
-        <f>IF(J16=0,"",IF(K16=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J16)),IF(L16&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L16),INDEX('2 Import devis'!$B$6:$B$29,J16))))</f>
+        <f>IF(J16=0,"",IF(K16=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J16)),IF(L16&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L16,2)),INDEX('2 Import devis'!$B$6:$B$29,J16))))</f>
         <v/>
       </c>
       <c r="D16" s="17">
@@ -1193,11 +1212,11 @@
         <v/>
       </c>
       <c r="E16" s="17">
-        <f>IF(K16=1,"",IF(L16&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L16)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L16)),"FR"))</f>
+        <f>IF(OR(J16=0,K16=1),"",IF(L16&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L16,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L16,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L16,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F16" s="18">
-        <f>IF(L16&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L16)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L16)),"")</f>
+        <f>IF(L16&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L16,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L16,3),1)),"")</f>
         <v/>
       </c>
       <c r="G16" s="19">
@@ -1221,26 +1240,30 @@
         <v/>
       </c>
       <c r="M16" s="20">
-        <f>IF(L16&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L16)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L16)),"")</f>
+        <f>IF(L16&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L16,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L16,20)),"")</f>
         <v/>
       </c>
       <c r="N16" s="20">
-        <f>IF(L16&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L16)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L16)),"")</f>
+        <f>IF(L16&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L16,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L16,23)),"")</f>
         <v/>
       </c>
       <c r="O16" s="20">
-        <f>IF(L16&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L16)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L16)),"")</f>
+        <f>IF(L16&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L16,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L16,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P16" s="20">
+        <f>IF(L16&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L16,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L16,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="17" ht="26" customHeight="1">
       <c r="A17" s="15">
-        <f>IF(L17&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L17),"")</f>
+        <f>IF(OR(J17=0,K17=1),"",COUNTIF(K$15:K17,0)-COUNTIF(J$15:J17,0))</f>
         <v/>
       </c>
       <c r="B17" s="15" t="n"/>
       <c r="C17" s="16">
-        <f>IF(J17=0,"",IF(K17=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J17)),IF(L17&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L17),INDEX('2 Import devis'!$B$6:$B$29,J17))))</f>
+        <f>IF(J17=0,"",IF(K17=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J17)),IF(L17&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L17,2)),INDEX('2 Import devis'!$B$6:$B$29,J17))))</f>
         <v/>
       </c>
       <c r="D17" s="17">
@@ -1248,11 +1271,11 @@
         <v/>
       </c>
       <c r="E17" s="17">
-        <f>IF(K17=1,"",IF(L17&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L17)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L17)),"FR"))</f>
+        <f>IF(OR(J17=0,K17=1),"",IF(L17&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L17,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L17,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L17,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F17" s="18">
-        <f>IF(L17&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L17)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L17)),"")</f>
+        <f>IF(L17&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L17,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L17,3),1)),"")</f>
         <v/>
       </c>
       <c r="G17" s="19">
@@ -1276,26 +1299,30 @@
         <v/>
       </c>
       <c r="M17" s="20">
-        <f>IF(L17&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L17)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L17)),"")</f>
+        <f>IF(L17&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L17,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L17,20)),"")</f>
         <v/>
       </c>
       <c r="N17" s="20">
-        <f>IF(L17&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L17)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L17)),"")</f>
+        <f>IF(L17&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L17,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L17,23)),"")</f>
         <v/>
       </c>
       <c r="O17" s="20">
-        <f>IF(L17&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L17)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L17)),"")</f>
+        <f>IF(L17&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L17,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L17,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P17" s="20">
+        <f>IF(L17&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L17,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L17,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="26" customHeight="1">
       <c r="A18" s="15">
-        <f>IF(L18&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L18),"")</f>
+        <f>IF(OR(J18=0,K18=1),"",COUNTIF(K$15:K18,0)-COUNTIF(J$15:J18,0))</f>
         <v/>
       </c>
       <c r="B18" s="15" t="n"/>
       <c r="C18" s="16">
-        <f>IF(J18=0,"",IF(K18=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J18)),IF(L18&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L18),INDEX('2 Import devis'!$B$6:$B$29,J18))))</f>
+        <f>IF(J18=0,"",IF(K18=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J18)),IF(L18&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L18,2)),INDEX('2 Import devis'!$B$6:$B$29,J18))))</f>
         <v/>
       </c>
       <c r="D18" s="17">
@@ -1303,11 +1330,11 @@
         <v/>
       </c>
       <c r="E18" s="17">
-        <f>IF(K18=1,"",IF(L18&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L18)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L18)),"FR"))</f>
+        <f>IF(OR(J18=0,K18=1),"",IF(L18&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L18,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L18,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L18,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F18" s="18">
-        <f>IF(L18&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L18)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L18)),"")</f>
+        <f>IF(L18&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L18,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L18,3),1)),"")</f>
         <v/>
       </c>
       <c r="G18" s="19">
@@ -1331,26 +1358,30 @@
         <v/>
       </c>
       <c r="M18" s="20">
-        <f>IF(L18&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L18)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L18)),"")</f>
+        <f>IF(L18&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L18,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L18,20)),"")</f>
         <v/>
       </c>
       <c r="N18" s="20">
-        <f>IF(L18&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L18)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L18)),"")</f>
+        <f>IF(L18&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L18,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L18,23)),"")</f>
         <v/>
       </c>
       <c r="O18" s="20">
-        <f>IF(L18&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L18)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L18)),"")</f>
+        <f>IF(L18&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L18,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L18,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P18" s="20">
+        <f>IF(L18&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L18,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L18,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="19" ht="26" customHeight="1">
       <c r="A19" s="15">
-        <f>IF(L19&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L19),"")</f>
+        <f>IF(OR(J19=0,K19=1),"",COUNTIF(K$15:K19,0)-COUNTIF(J$15:J19,0))</f>
         <v/>
       </c>
       <c r="B19" s="15" t="n"/>
       <c r="C19" s="16">
-        <f>IF(J19=0,"",IF(K19=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J19)),IF(L19&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L19),INDEX('2 Import devis'!$B$6:$B$29,J19))))</f>
+        <f>IF(J19=0,"",IF(K19=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J19)),IF(L19&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L19,2)),INDEX('2 Import devis'!$B$6:$B$29,J19))))</f>
         <v/>
       </c>
       <c r="D19" s="17">
@@ -1358,11 +1389,11 @@
         <v/>
       </c>
       <c r="E19" s="17">
-        <f>IF(K19=1,"",IF(L19&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L19)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L19)),"FR"))</f>
+        <f>IF(OR(J19=0,K19=1),"",IF(L19&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L19,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L19,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L19,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F19" s="18">
-        <f>IF(L19&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L19)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L19)),"")</f>
+        <f>IF(L19&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L19,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L19,3),1)),"")</f>
         <v/>
       </c>
       <c r="G19" s="19">
@@ -1386,26 +1417,30 @@
         <v/>
       </c>
       <c r="M19" s="20">
-        <f>IF(L19&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L19)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L19)),"")</f>
+        <f>IF(L19&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L19,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L19,20)),"")</f>
         <v/>
       </c>
       <c r="N19" s="20">
-        <f>IF(L19&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L19)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L19)),"")</f>
+        <f>IF(L19&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L19,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L19,23)),"")</f>
         <v/>
       </c>
       <c r="O19" s="20">
-        <f>IF(L19&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L19)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L19)),"")</f>
+        <f>IF(L19&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L19,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L19,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P19" s="20">
+        <f>IF(L19&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L19,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L19,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="20" hidden="1" ht="26" customHeight="1">
       <c r="A20" s="15">
-        <f>IF(L20&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L20),"")</f>
+        <f>IF(OR(J20=0,K20=1),"",COUNTIF(K$15:K20,0)-COUNTIF(J$15:J20,0))</f>
         <v/>
       </c>
       <c r="B20" s="15" t="n"/>
       <c r="C20" s="16">
-        <f>IF(J20=0,"",IF(K20=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J20)),IF(L20&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L20),INDEX('2 Import devis'!$B$6:$B$29,J20))))</f>
+        <f>IF(J20=0,"",IF(K20=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J20)),IF(L20&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L20,2)),INDEX('2 Import devis'!$B$6:$B$29,J20))))</f>
         <v/>
       </c>
       <c r="D20" s="17">
@@ -1413,11 +1448,11 @@
         <v/>
       </c>
       <c r="E20" s="17">
-        <f>IF(K20=1,"",IF(L20&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L20)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L20)),"FR"))</f>
+        <f>IF(OR(J20=0,K20=1),"",IF(L20&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L20,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L20,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L20,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F20" s="18">
-        <f>IF(L20&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L20)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L20)),"")</f>
+        <f>IF(L20&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L20,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L20,3),1)),"")</f>
         <v/>
       </c>
       <c r="G20" s="19">
@@ -1441,26 +1476,30 @@
         <v/>
       </c>
       <c r="M20" s="20">
-        <f>IF(L20&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L20)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L20)),"")</f>
+        <f>IF(L20&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L20,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L20,20)),"")</f>
         <v/>
       </c>
       <c r="N20" s="20">
-        <f>IF(L20&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L20)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L20)),"")</f>
+        <f>IF(L20&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L20,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L20,23)),"")</f>
         <v/>
       </c>
       <c r="O20" s="20">
-        <f>IF(L20&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L20)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L20)),"")</f>
+        <f>IF(L20&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L20,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L20,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P20" s="20">
+        <f>IF(L20&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L20,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L20,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="21" hidden="1" ht="26" customHeight="1">
       <c r="A21" s="15">
-        <f>IF(L21&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L21),"")</f>
+        <f>IF(OR(J21=0,K21=1),"",COUNTIF(K$15:K21,0)-COUNTIF(J$15:J21,0))</f>
         <v/>
       </c>
       <c r="B21" s="15" t="n"/>
       <c r="C21" s="16">
-        <f>IF(J21=0,"",IF(K21=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J21)),IF(L21&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L21),INDEX('2 Import devis'!$B$6:$B$29,J21))))</f>
+        <f>IF(J21=0,"",IF(K21=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J21)),IF(L21&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L21,2)),INDEX('2 Import devis'!$B$6:$B$29,J21))))</f>
         <v/>
       </c>
       <c r="D21" s="17">
@@ -1468,11 +1507,11 @@
         <v/>
       </c>
       <c r="E21" s="17">
-        <f>IF(K21=1,"",IF(L21&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L21)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L21)),"FR"))</f>
+        <f>IF(OR(J21=0,K21=1),"",IF(L21&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L21,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L21,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L21,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F21" s="18">
-        <f>IF(L21&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L21)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L21)),"")</f>
+        <f>IF(L21&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L21,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L21,3),1)),"")</f>
         <v/>
       </c>
       <c r="G21" s="19">
@@ -1496,26 +1535,30 @@
         <v/>
       </c>
       <c r="M21" s="20">
-        <f>IF(L21&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L21)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L21)),"")</f>
+        <f>IF(L21&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L21,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L21,20)),"")</f>
         <v/>
       </c>
       <c r="N21" s="20">
-        <f>IF(L21&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L21)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L21)),"")</f>
+        <f>IF(L21&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L21,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L21,23)),"")</f>
         <v/>
       </c>
       <c r="O21" s="20">
-        <f>IF(L21&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L21)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L21)),"")</f>
+        <f>IF(L21&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L21,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L21,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P21" s="20">
+        <f>IF(L21&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L21,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L21,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="22" hidden="1" ht="26" customHeight="1">
       <c r="A22" s="15">
-        <f>IF(L22&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L22),"")</f>
+        <f>IF(OR(J22=0,K22=1),"",COUNTIF(K$15:K22,0)-COUNTIF(J$15:J22,0))</f>
         <v/>
       </c>
       <c r="B22" s="15" t="n"/>
       <c r="C22" s="16">
-        <f>IF(J22=0,"",IF(K22=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J22)),IF(L22&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L22),INDEX('2 Import devis'!$B$6:$B$29,J22))))</f>
+        <f>IF(J22=0,"",IF(K22=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J22)),IF(L22&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L22,2)),INDEX('2 Import devis'!$B$6:$B$29,J22))))</f>
         <v/>
       </c>
       <c r="D22" s="17">
@@ -1523,11 +1566,11 @@
         <v/>
       </c>
       <c r="E22" s="17">
-        <f>IF(K22=1,"",IF(L22&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L22)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L22)),"FR"))</f>
+        <f>IF(OR(J22=0,K22=1),"",IF(L22&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L22,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L22,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L22,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F22" s="18">
-        <f>IF(L22&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L22)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L22)),"")</f>
+        <f>IF(L22&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L22,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L22,3),1)),"")</f>
         <v/>
       </c>
       <c r="G22" s="19">
@@ -1551,26 +1594,30 @@
         <v/>
       </c>
       <c r="M22" s="20">
-        <f>IF(L22&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L22)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L22)),"")</f>
+        <f>IF(L22&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L22,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L22,20)),"")</f>
         <v/>
       </c>
       <c r="N22" s="20">
-        <f>IF(L22&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L22)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L22)),"")</f>
+        <f>IF(L22&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L22,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L22,23)),"")</f>
         <v/>
       </c>
       <c r="O22" s="20">
-        <f>IF(L22&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L22)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L22)),"")</f>
+        <f>IF(L22&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L22,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L22,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P22" s="20">
+        <f>IF(L22&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L22,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L22,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="23" hidden="1" ht="26" customHeight="1">
       <c r="A23" s="15">
-        <f>IF(L23&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L23),"")</f>
+        <f>IF(OR(J23=0,K23=1),"",COUNTIF(K$15:K23,0)-COUNTIF(J$15:J23,0))</f>
         <v/>
       </c>
       <c r="B23" s="15" t="n"/>
       <c r="C23" s="16">
-        <f>IF(J23=0,"",IF(K23=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J23)),IF(L23&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L23),INDEX('2 Import devis'!$B$6:$B$29,J23))))</f>
+        <f>IF(J23=0,"",IF(K23=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J23)),IF(L23&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L23,2)),INDEX('2 Import devis'!$B$6:$B$29,J23))))</f>
         <v/>
       </c>
       <c r="D23" s="17">
@@ -1578,11 +1625,11 @@
         <v/>
       </c>
       <c r="E23" s="17">
-        <f>IF(K23=1,"",IF(L23&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L23)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L23)),"FR"))</f>
+        <f>IF(OR(J23=0,K23=1),"",IF(L23&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L23,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L23,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L23,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F23" s="18">
-        <f>IF(L23&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L23)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L23)),"")</f>
+        <f>IF(L23&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L23,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L23,3),1)),"")</f>
         <v/>
       </c>
       <c r="G23" s="19">
@@ -1606,26 +1653,30 @@
         <v/>
       </c>
       <c r="M23" s="20">
-        <f>IF(L23&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L23)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L23)),"")</f>
+        <f>IF(L23&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L23,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L23,20)),"")</f>
         <v/>
       </c>
       <c r="N23" s="20">
-        <f>IF(L23&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L23)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L23)),"")</f>
+        <f>IF(L23&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L23,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L23,23)),"")</f>
         <v/>
       </c>
       <c r="O23" s="20">
-        <f>IF(L23&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L23)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L23)),"")</f>
+        <f>IF(L23&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L23,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L23,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P23" s="20">
+        <f>IF(L23&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L23,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L23,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="24" hidden="1" ht="26" customHeight="1">
       <c r="A24" s="15">
-        <f>IF(L24&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L24),"")</f>
+        <f>IF(OR(J24=0,K24=1),"",COUNTIF(K$15:K24,0)-COUNTIF(J$15:J24,0))</f>
         <v/>
       </c>
       <c r="B24" s="15" t="n"/>
       <c r="C24" s="16">
-        <f>IF(J24=0,"",IF(K24=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J24)),IF(L24&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L24),INDEX('2 Import devis'!$B$6:$B$29,J24))))</f>
+        <f>IF(J24=0,"",IF(K24=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J24)),IF(L24&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L24,2)),INDEX('2 Import devis'!$B$6:$B$29,J24))))</f>
         <v/>
       </c>
       <c r="D24" s="17">
@@ -1633,11 +1684,11 @@
         <v/>
       </c>
       <c r="E24" s="17">
-        <f>IF(K24=1,"",IF(L24&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L24)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L24)),"FR"))</f>
+        <f>IF(OR(J24=0,K24=1),"",IF(L24&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L24,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L24,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L24,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F24" s="18">
-        <f>IF(L24&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L24)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L24)),"")</f>
+        <f>IF(L24&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L24,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L24,3),1)),"")</f>
         <v/>
       </c>
       <c r="G24" s="19">
@@ -1661,26 +1712,30 @@
         <v/>
       </c>
       <c r="M24" s="20">
-        <f>IF(L24&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L24)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L24)),"")</f>
+        <f>IF(L24&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L24,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L24,20)),"")</f>
         <v/>
       </c>
       <c r="N24" s="20">
-        <f>IF(L24&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L24)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L24)),"")</f>
+        <f>IF(L24&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L24,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L24,23)),"")</f>
         <v/>
       </c>
       <c r="O24" s="20">
-        <f>IF(L24&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L24)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L24)),"")</f>
+        <f>IF(L24&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L24,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L24,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P24" s="20">
+        <f>IF(L24&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L24,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L24,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="25" hidden="1" ht="26" customHeight="1">
       <c r="A25" s="15">
-        <f>IF(L25&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L25),"")</f>
+        <f>IF(OR(J25=0,K25=1),"",COUNTIF(K$15:K25,0)-COUNTIF(J$15:J25,0))</f>
         <v/>
       </c>
       <c r="B25" s="15" t="n"/>
       <c r="C25" s="16">
-        <f>IF(J25=0,"",IF(K25=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J25)),IF(L25&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L25),INDEX('2 Import devis'!$B$6:$B$29,J25))))</f>
+        <f>IF(J25=0,"",IF(K25=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J25)),IF(L25&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L25,2)),INDEX('2 Import devis'!$B$6:$B$29,J25))))</f>
         <v/>
       </c>
       <c r="D25" s="17">
@@ -1688,11 +1743,11 @@
         <v/>
       </c>
       <c r="E25" s="17">
-        <f>IF(K25=1,"",IF(L25&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L25)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L25)),"FR"))</f>
+        <f>IF(OR(J25=0,K25=1),"",IF(L25&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L25,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L25,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L25,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F25" s="18">
-        <f>IF(L25&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L25)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L25)),"")</f>
+        <f>IF(L25&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L25,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L25,3),1)),"")</f>
         <v/>
       </c>
       <c r="G25" s="19">
@@ -1716,26 +1771,30 @@
         <v/>
       </c>
       <c r="M25" s="20">
-        <f>IF(L25&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L25)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L25)),"")</f>
+        <f>IF(L25&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L25,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L25,20)),"")</f>
         <v/>
       </c>
       <c r="N25" s="20">
-        <f>IF(L25&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L25)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L25)),"")</f>
+        <f>IF(L25&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L25,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L25,23)),"")</f>
         <v/>
       </c>
       <c r="O25" s="20">
-        <f>IF(L25&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L25)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L25)),"")</f>
+        <f>IF(L25&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L25,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L25,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P25" s="20">
+        <f>IF(L25&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L25,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L25,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="26" hidden="1" ht="26" customHeight="1">
       <c r="A26" s="15">
-        <f>IF(L26&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L26),"")</f>
+        <f>IF(OR(J26=0,K26=1),"",COUNTIF(K$15:K26,0)-COUNTIF(J$15:J26,0))</f>
         <v/>
       </c>
       <c r="B26" s="15" t="n"/>
       <c r="C26" s="16">
-        <f>IF(J26=0,"",IF(K26=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J26)),IF(L26&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L26),INDEX('2 Import devis'!$B$6:$B$29,J26))))</f>
+        <f>IF(J26=0,"",IF(K26=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J26)),IF(L26&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L26,2)),INDEX('2 Import devis'!$B$6:$B$29,J26))))</f>
         <v/>
       </c>
       <c r="D26" s="17">
@@ -1743,11 +1802,11 @@
         <v/>
       </c>
       <c r="E26" s="17">
-        <f>IF(K26=1,"",IF(L26&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L26)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L26)),"FR"))</f>
+        <f>IF(OR(J26=0,K26=1),"",IF(L26&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L26,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L26,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L26,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F26" s="18">
-        <f>IF(L26&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L26)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L26)),"")</f>
+        <f>IF(L26&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L26,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L26,3),1)),"")</f>
         <v/>
       </c>
       <c r="G26" s="19">
@@ -1771,26 +1830,30 @@
         <v/>
       </c>
       <c r="M26" s="20">
-        <f>IF(L26&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L26)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L26)),"")</f>
+        <f>IF(L26&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L26,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L26,20)),"")</f>
         <v/>
       </c>
       <c r="N26" s="20">
-        <f>IF(L26&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L26)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L26)),"")</f>
+        <f>IF(L26&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L26,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L26,23)),"")</f>
         <v/>
       </c>
       <c r="O26" s="20">
-        <f>IF(L26&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L26)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L26)),"")</f>
+        <f>IF(L26&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L26,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L26,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P26" s="20">
+        <f>IF(L26&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L26,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L26,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="27" hidden="1" ht="26" customHeight="1">
       <c r="A27" s="15">
-        <f>IF(L27&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L27),"")</f>
+        <f>IF(OR(J27=0,K27=1),"",COUNTIF(K$15:K27,0)-COUNTIF(J$15:J27,0))</f>
         <v/>
       </c>
       <c r="B27" s="15" t="n"/>
       <c r="C27" s="16">
-        <f>IF(J27=0,"",IF(K27=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J27)),IF(L27&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L27),INDEX('2 Import devis'!$B$6:$B$29,J27))))</f>
+        <f>IF(J27=0,"",IF(K27=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J27)),IF(L27&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L27,2)),INDEX('2 Import devis'!$B$6:$B$29,J27))))</f>
         <v/>
       </c>
       <c r="D27" s="17">
@@ -1798,11 +1861,11 @@
         <v/>
       </c>
       <c r="E27" s="17">
-        <f>IF(K27=1,"",IF(L27&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L27)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L27)),"FR"))</f>
+        <f>IF(OR(J27=0,K27=1),"",IF(L27&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L27,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L27,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L27,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F27" s="18">
-        <f>IF(L27&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L27)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L27)),"")</f>
+        <f>IF(L27&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L27,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L27,3),1)),"")</f>
         <v/>
       </c>
       <c r="G27" s="19">
@@ -1826,26 +1889,30 @@
         <v/>
       </c>
       <c r="M27" s="20">
-        <f>IF(L27&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L27)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L27)),"")</f>
+        <f>IF(L27&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L27,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L27,20)),"")</f>
         <v/>
       </c>
       <c r="N27" s="20">
-        <f>IF(L27&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L27)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L27)),"")</f>
+        <f>IF(L27&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L27,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L27,23)),"")</f>
         <v/>
       </c>
       <c r="O27" s="20">
-        <f>IF(L27&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L27)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L27)),"")</f>
+        <f>IF(L27&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L27,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L27,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P27" s="20">
+        <f>IF(L27&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L27,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L27,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="28" hidden="1" ht="26" customHeight="1">
       <c r="A28" s="15">
-        <f>IF(L28&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L28),"")</f>
+        <f>IF(OR(J28=0,K28=1),"",COUNTIF(K$15:K28,0)-COUNTIF(J$15:J28,0))</f>
         <v/>
       </c>
       <c r="B28" s="15" t="n"/>
       <c r="C28" s="16">
-        <f>IF(J28=0,"",IF(K28=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J28)),IF(L28&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L28),INDEX('2 Import devis'!$B$6:$B$29,J28))))</f>
+        <f>IF(J28=0,"",IF(K28=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J28)),IF(L28&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L28,2)),INDEX('2 Import devis'!$B$6:$B$29,J28))))</f>
         <v/>
       </c>
       <c r="D28" s="17">
@@ -1853,11 +1920,11 @@
         <v/>
       </c>
       <c r="E28" s="17">
-        <f>IF(K28=1,"",IF(L28&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L28)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L28)),"FR"))</f>
+        <f>IF(OR(J28=0,K28=1),"",IF(L28&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L28,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L28,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L28,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F28" s="18">
-        <f>IF(L28&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L28)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L28)),"")</f>
+        <f>IF(L28&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L28,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L28,3),1)),"")</f>
         <v/>
       </c>
       <c r="G28" s="19">
@@ -1881,26 +1948,30 @@
         <v/>
       </c>
       <c r="M28" s="20">
-        <f>IF(L28&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L28)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L28)),"")</f>
+        <f>IF(L28&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L28,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L28,20)),"")</f>
         <v/>
       </c>
       <c r="N28" s="20">
-        <f>IF(L28&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L28)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L28)),"")</f>
+        <f>IF(L28&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L28,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L28,23)),"")</f>
         <v/>
       </c>
       <c r="O28" s="20">
-        <f>IF(L28&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L28)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L28)),"")</f>
+        <f>IF(L28&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L28,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L28,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P28" s="20">
+        <f>IF(L28&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L28,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L28,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="29" hidden="1" ht="26" customHeight="1">
       <c r="A29" s="15">
-        <f>IF(L29&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L29),"")</f>
+        <f>IF(OR(J29=0,K29=1),"",COUNTIF(K$15:K29,0)-COUNTIF(J$15:J29,0))</f>
         <v/>
       </c>
       <c r="B29" s="15" t="n"/>
       <c r="C29" s="16">
-        <f>IF(J29=0,"",IF(K29=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J29)),IF(L29&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L29),INDEX('2 Import devis'!$B$6:$B$29,J29))))</f>
+        <f>IF(J29=0,"",IF(K29=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J29)),IF(L29&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L29,2)),INDEX('2 Import devis'!$B$6:$B$29,J29))))</f>
         <v/>
       </c>
       <c r="D29" s="17">
@@ -1908,11 +1979,11 @@
         <v/>
       </c>
       <c r="E29" s="17">
-        <f>IF(K29=1,"",IF(L29&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L29)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L29)),"FR"))</f>
+        <f>IF(OR(J29=0,K29=1),"",IF(L29&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L29,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L29,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L29,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F29" s="18">
-        <f>IF(L29&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L29)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L29)),"")</f>
+        <f>IF(L29&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L29,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L29,3),1)),"")</f>
         <v/>
       </c>
       <c r="G29" s="19">
@@ -1936,26 +2007,30 @@
         <v/>
       </c>
       <c r="M29" s="20">
-        <f>IF(L29&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L29)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L29)),"")</f>
+        <f>IF(L29&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L29,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L29,20)),"")</f>
         <v/>
       </c>
       <c r="N29" s="20">
-        <f>IF(L29&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L29)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L29)),"")</f>
+        <f>IF(L29&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L29,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L29,23)),"")</f>
         <v/>
       </c>
       <c r="O29" s="20">
-        <f>IF(L29&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L29)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L29)),"")</f>
+        <f>IF(L29&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L29,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L29,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P29" s="20">
+        <f>IF(L29&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L29,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L29,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="30" hidden="1" ht="26" customHeight="1">
       <c r="A30" s="15">
-        <f>IF(L30&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L30),"")</f>
+        <f>IF(OR(J30=0,K30=1),"",COUNTIF(K$15:K30,0)-COUNTIF(J$15:J30,0))</f>
         <v/>
       </c>
       <c r="B30" s="15" t="n"/>
       <c r="C30" s="16">
-        <f>IF(J30=0,"",IF(K30=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J30)),IF(L30&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L30),INDEX('2 Import devis'!$B$6:$B$29,J30))))</f>
+        <f>IF(J30=0,"",IF(K30=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J30)),IF(L30&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L30,2)),INDEX('2 Import devis'!$B$6:$B$29,J30))))</f>
         <v/>
       </c>
       <c r="D30" s="17">
@@ -1963,11 +2038,11 @@
         <v/>
       </c>
       <c r="E30" s="17">
-        <f>IF(K30=1,"",IF(L30&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L30)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L30)),"FR"))</f>
+        <f>IF(OR(J30=0,K30=1),"",IF(L30&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L30,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L30,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L30,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F30" s="18">
-        <f>IF(L30&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L30)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L30)),"")</f>
+        <f>IF(L30&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L30,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L30,3),1)),"")</f>
         <v/>
       </c>
       <c r="G30" s="19">
@@ -1991,26 +2066,30 @@
         <v/>
       </c>
       <c r="M30" s="20">
-        <f>IF(L30&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L30)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L30)),"")</f>
+        <f>IF(L30&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L30,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L30,20)),"")</f>
         <v/>
       </c>
       <c r="N30" s="20">
-        <f>IF(L30&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L30)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L30)),"")</f>
+        <f>IF(L30&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L30,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L30,23)),"")</f>
         <v/>
       </c>
       <c r="O30" s="20">
-        <f>IF(L30&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L30)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L30)),"")</f>
+        <f>IF(L30&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L30,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L30,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P30" s="20">
+        <f>IF(L30&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L30,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L30,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="31" hidden="1" ht="26" customHeight="1">
       <c r="A31" s="15">
-        <f>IF(L31&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L31),"")</f>
+        <f>IF(OR(J31=0,K31=1),"",COUNTIF(K$15:K31,0)-COUNTIF(J$15:J31,0))</f>
         <v/>
       </c>
       <c r="B31" s="15" t="n"/>
       <c r="C31" s="16">
-        <f>IF(J31=0,"",IF(K31=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J31)),IF(L31&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L31),INDEX('2 Import devis'!$B$6:$B$29,J31))))</f>
+        <f>IF(J31=0,"",IF(K31=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J31)),IF(L31&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L31,2)),INDEX('2 Import devis'!$B$6:$B$29,J31))))</f>
         <v/>
       </c>
       <c r="D31" s="17">
@@ -2018,11 +2097,11 @@
         <v/>
       </c>
       <c r="E31" s="17">
-        <f>IF(K31=1,"",IF(L31&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L31)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L31)),"FR"))</f>
+        <f>IF(OR(J31=0,K31=1),"",IF(L31&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L31,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L31,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L31,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F31" s="18">
-        <f>IF(L31&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L31)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L31)),"")</f>
+        <f>IF(L31&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L31,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L31,3),1)),"")</f>
         <v/>
       </c>
       <c r="G31" s="19">
@@ -2046,26 +2125,30 @@
         <v/>
       </c>
       <c r="M31" s="20">
-        <f>IF(L31&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L31)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L31)),"")</f>
+        <f>IF(L31&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L31,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L31,20)),"")</f>
         <v/>
       </c>
       <c r="N31" s="20">
-        <f>IF(L31&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L31)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L31)),"")</f>
+        <f>IF(L31&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L31,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L31,23)),"")</f>
         <v/>
       </c>
       <c r="O31" s="20">
-        <f>IF(L31&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L31)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L31)),"")</f>
+        <f>IF(L31&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L31,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L31,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P31" s="20">
+        <f>IF(L31&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L31,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L31,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="32" hidden="1" ht="26" customHeight="1">
       <c r="A32" s="15">
-        <f>IF(L32&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L32),"")</f>
+        <f>IF(OR(J32=0,K32=1),"",COUNTIF(K$15:K32,0)-COUNTIF(J$15:J32,0))</f>
         <v/>
       </c>
       <c r="B32" s="15" t="n"/>
       <c r="C32" s="16">
-        <f>IF(J32=0,"",IF(K32=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J32)),IF(L32&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L32),INDEX('2 Import devis'!$B$6:$B$29,J32))))</f>
+        <f>IF(J32=0,"",IF(K32=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J32)),IF(L32&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L32,2)),INDEX('2 Import devis'!$B$6:$B$29,J32))))</f>
         <v/>
       </c>
       <c r="D32" s="17">
@@ -2073,11 +2156,11 @@
         <v/>
       </c>
       <c r="E32" s="17">
-        <f>IF(K32=1,"",IF(L32&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L32)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L32)),"FR"))</f>
+        <f>IF(OR(J32=0,K32=1),"",IF(L32&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L32,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L32,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L32,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F32" s="18">
-        <f>IF(L32&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L32)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L32)),"")</f>
+        <f>IF(L32&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L32,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L32,3),1)),"")</f>
         <v/>
       </c>
       <c r="G32" s="19">
@@ -2101,26 +2184,30 @@
         <v/>
       </c>
       <c r="M32" s="20">
-        <f>IF(L32&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L32)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L32)),"")</f>
+        <f>IF(L32&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L32,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L32,20)),"")</f>
         <v/>
       </c>
       <c r="N32" s="20">
-        <f>IF(L32&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L32)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L32)),"")</f>
+        <f>IF(L32&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L32,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L32,23)),"")</f>
         <v/>
       </c>
       <c r="O32" s="20">
-        <f>IF(L32&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L32)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L32)),"")</f>
+        <f>IF(L32&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L32,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L32,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P32" s="20">
+        <f>IF(L32&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L32,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L32,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="33" hidden="1" ht="26" customHeight="1">
       <c r="A33" s="15">
-        <f>IF(L33&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L33),"")</f>
+        <f>IF(OR(J33=0,K33=1),"",COUNTIF(K$15:K33,0)-COUNTIF(J$15:J33,0))</f>
         <v/>
       </c>
       <c r="B33" s="15" t="n"/>
       <c r="C33" s="16">
-        <f>IF(J33=0,"",IF(K33=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J33)),IF(L33&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L33),INDEX('2 Import devis'!$B$6:$B$29,J33))))</f>
+        <f>IF(J33=0,"",IF(K33=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J33)),IF(L33&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L33,2)),INDEX('2 Import devis'!$B$6:$B$29,J33))))</f>
         <v/>
       </c>
       <c r="D33" s="17">
@@ -2128,11 +2215,11 @@
         <v/>
       </c>
       <c r="E33" s="17">
-        <f>IF(K33=1,"",IF(L33&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L33)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L33)),"FR"))</f>
+        <f>IF(OR(J33=0,K33=1),"",IF(L33&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L33,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L33,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L33,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F33" s="18">
-        <f>IF(L33&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L33)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L33)),"")</f>
+        <f>IF(L33&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L33,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L33,3),1)),"")</f>
         <v/>
       </c>
       <c r="G33" s="19">
@@ -2156,26 +2243,30 @@
         <v/>
       </c>
       <c r="M33" s="20">
-        <f>IF(L33&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L33)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L33)),"")</f>
+        <f>IF(L33&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L33,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L33,20)),"")</f>
         <v/>
       </c>
       <c r="N33" s="20">
-        <f>IF(L33&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L33)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L33)),"")</f>
+        <f>IF(L33&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L33,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L33,23)),"")</f>
         <v/>
       </c>
       <c r="O33" s="20">
-        <f>IF(L33&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L33)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L33)),"")</f>
+        <f>IF(L33&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L33,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L33,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P33" s="20">
+        <f>IF(L33&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L33,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L33,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="34" hidden="1" ht="26" customHeight="1">
       <c r="A34" s="15">
-        <f>IF(L34&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L34),"")</f>
+        <f>IF(OR(J34=0,K34=1),"",COUNTIF(K$15:K34,0)-COUNTIF(J$15:J34,0))</f>
         <v/>
       </c>
       <c r="B34" s="15" t="n"/>
       <c r="C34" s="16">
-        <f>IF(J34=0,"",IF(K34=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J34)),IF(L34&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L34),INDEX('2 Import devis'!$B$6:$B$29,J34))))</f>
+        <f>IF(J34=0,"",IF(K34=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J34)),IF(L34&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L34,2)),INDEX('2 Import devis'!$B$6:$B$29,J34))))</f>
         <v/>
       </c>
       <c r="D34" s="17">
@@ -2183,11 +2274,11 @@
         <v/>
       </c>
       <c r="E34" s="17">
-        <f>IF(K34=1,"",IF(L34&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L34)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L34)),"FR"))</f>
+        <f>IF(OR(J34=0,K34=1),"",IF(L34&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L34,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L34,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L34,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F34" s="18">
-        <f>IF(L34&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L34)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L34)),"")</f>
+        <f>IF(L34&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L34,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L34,3),1)),"")</f>
         <v/>
       </c>
       <c r="G34" s="19">
@@ -2211,26 +2302,30 @@
         <v/>
       </c>
       <c r="M34" s="20">
-        <f>IF(L34&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L34)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L34)),"")</f>
+        <f>IF(L34&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L34,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L34,20)),"")</f>
         <v/>
       </c>
       <c r="N34" s="20">
-        <f>IF(L34&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L34)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L34)),"")</f>
+        <f>IF(L34&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L34,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L34,23)),"")</f>
         <v/>
       </c>
       <c r="O34" s="20">
-        <f>IF(L34&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L34)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L34)),"")</f>
+        <f>IF(L34&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L34,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L34,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P34" s="20">
+        <f>IF(L34&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L34,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L34,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="35" hidden="1" ht="26" customHeight="1">
       <c r="A35" s="15">
-        <f>IF(L35&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L35),"")</f>
+        <f>IF(OR(J35=0,K35=1),"",COUNTIF(K$15:K35,0)-COUNTIF(J$15:J35,0))</f>
         <v/>
       </c>
       <c r="B35" s="15" t="n"/>
       <c r="C35" s="16">
-        <f>IF(J35=0,"",IF(K35=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J35)),IF(L35&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L35),INDEX('2 Import devis'!$B$6:$B$29,J35))))</f>
+        <f>IF(J35=0,"",IF(K35=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J35)),IF(L35&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L35,2)),INDEX('2 Import devis'!$B$6:$B$29,J35))))</f>
         <v/>
       </c>
       <c r="D35" s="17">
@@ -2238,11 +2333,11 @@
         <v/>
       </c>
       <c r="E35" s="17">
-        <f>IF(K35=1,"",IF(L35&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L35)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L35)),"FR"))</f>
+        <f>IF(OR(J35=0,K35=1),"",IF(L35&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L35,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L35,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L35,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F35" s="18">
-        <f>IF(L35&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L35)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L35)),"")</f>
+        <f>IF(L35&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L35,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L35,3),1)),"")</f>
         <v/>
       </c>
       <c r="G35" s="19">
@@ -2266,26 +2361,30 @@
         <v/>
       </c>
       <c r="M35" s="20">
-        <f>IF(L35&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L35)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L35)),"")</f>
+        <f>IF(L35&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L35,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L35,20)),"")</f>
         <v/>
       </c>
       <c r="N35" s="20">
-        <f>IF(L35&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L35)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L35)),"")</f>
+        <f>IF(L35&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L35,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L35,23)),"")</f>
         <v/>
       </c>
       <c r="O35" s="20">
-        <f>IF(L35&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L35)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L35)),"")</f>
+        <f>IF(L35&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L35,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L35,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P35" s="20">
+        <f>IF(L35&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L35,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L35,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="36" hidden="1" ht="26" customHeight="1">
       <c r="A36" s="15">
-        <f>IF(L36&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L36),"")</f>
+        <f>IF(OR(J36=0,K36=1),"",COUNTIF(K$15:K36,0)-COUNTIF(J$15:J36,0))</f>
         <v/>
       </c>
       <c r="B36" s="15" t="n"/>
       <c r="C36" s="16">
-        <f>IF(J36=0,"",IF(K36=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J36)),IF(L36&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L36),INDEX('2 Import devis'!$B$6:$B$29,J36))))</f>
+        <f>IF(J36=0,"",IF(K36=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J36)),IF(L36&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L36,2)),INDEX('2 Import devis'!$B$6:$B$29,J36))))</f>
         <v/>
       </c>
       <c r="D36" s="17">
@@ -2293,11 +2392,11 @@
         <v/>
       </c>
       <c r="E36" s="17">
-        <f>IF(K36=1,"",IF(L36&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L36)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L36)),"FR"))</f>
+        <f>IF(OR(J36=0,K36=1),"",IF(L36&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L36,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L36,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L36,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F36" s="18">
-        <f>IF(L36&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L36)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L36)),"")</f>
+        <f>IF(L36&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L36,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L36,3),1)),"")</f>
         <v/>
       </c>
       <c r="G36" s="19">
@@ -2321,26 +2420,30 @@
         <v/>
       </c>
       <c r="M36" s="20">
-        <f>IF(L36&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L36)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L36)),"")</f>
+        <f>IF(L36&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L36,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L36,20)),"")</f>
         <v/>
       </c>
       <c r="N36" s="20">
-        <f>IF(L36&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L36)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L36)),"")</f>
+        <f>IF(L36&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L36,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L36,23)),"")</f>
         <v/>
       </c>
       <c r="O36" s="20">
-        <f>IF(L36&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L36)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L36)),"")</f>
+        <f>IF(L36&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L36,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L36,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P36" s="20">
+        <f>IF(L36&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L36,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L36,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="37" hidden="1" ht="26" customHeight="1">
       <c r="A37" s="15">
-        <f>IF(L37&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L37),"")</f>
+        <f>IF(OR(J37=0,K37=1),"",COUNTIF(K$15:K37,0)-COUNTIF(J$15:J37,0))</f>
         <v/>
       </c>
       <c r="B37" s="15" t="n"/>
       <c r="C37" s="16">
-        <f>IF(J37=0,"",IF(K37=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J37)),IF(L37&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L37),INDEX('2 Import devis'!$B$6:$B$29,J37))))</f>
+        <f>IF(J37=0,"",IF(K37=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J37)),IF(L37&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L37,2)),INDEX('2 Import devis'!$B$6:$B$29,J37))))</f>
         <v/>
       </c>
       <c r="D37" s="17">
@@ -2348,11 +2451,11 @@
         <v/>
       </c>
       <c r="E37" s="17">
-        <f>IF(K37=1,"",IF(L37&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L37)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L37)),"FR"))</f>
+        <f>IF(OR(J37=0,K37=1),"",IF(L37&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L37,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L37,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L37,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F37" s="18">
-        <f>IF(L37&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L37)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L37)),"")</f>
+        <f>IF(L37&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L37,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L37,3),1)),"")</f>
         <v/>
       </c>
       <c r="G37" s="19">
@@ -2376,26 +2479,30 @@
         <v/>
       </c>
       <c r="M37" s="20">
-        <f>IF(L37&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L37)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L37)),"")</f>
+        <f>IF(L37&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L37,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L37,20)),"")</f>
         <v/>
       </c>
       <c r="N37" s="20">
-        <f>IF(L37&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L37)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L37)),"")</f>
+        <f>IF(L37&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L37,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L37,23)),"")</f>
         <v/>
       </c>
       <c r="O37" s="20">
-        <f>IF(L37&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L37)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L37)),"")</f>
+        <f>IF(L37&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L37,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L37,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P37" s="20">
+        <f>IF(L37&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L37,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L37,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="38" hidden="1" ht="26" customHeight="1">
       <c r="A38" s="15">
-        <f>IF(L38&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L38),"")</f>
+        <f>IF(OR(J38=0,K38=1),"",COUNTIF(K$15:K38,0)-COUNTIF(J$15:J38,0))</f>
         <v/>
       </c>
       <c r="B38" s="15" t="n"/>
       <c r="C38" s="16">
-        <f>IF(J38=0,"",IF(K38=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J38)),IF(L38&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L38),INDEX('2 Import devis'!$B$6:$B$29,J38))))</f>
+        <f>IF(J38=0,"",IF(K38=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J38)),IF(L38&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L38,2)),INDEX('2 Import devis'!$B$6:$B$29,J38))))</f>
         <v/>
       </c>
       <c r="D38" s="17">
@@ -2403,11 +2510,11 @@
         <v/>
       </c>
       <c r="E38" s="17">
-        <f>IF(K38=1,"",IF(L38&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L38)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L38)),"FR"))</f>
+        <f>IF(OR(J38=0,K38=1),"",IF(L38&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L38,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L38,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L38,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F38" s="18">
-        <f>IF(L38&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L38)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L38)),"")</f>
+        <f>IF(L38&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L38,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L38,3),1)),"")</f>
         <v/>
       </c>
       <c r="G38" s="19">
@@ -2431,26 +2538,30 @@
         <v/>
       </c>
       <c r="M38" s="20">
-        <f>IF(L38&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L38)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L38)),"")</f>
+        <f>IF(L38&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L38,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L38,20)),"")</f>
         <v/>
       </c>
       <c r="N38" s="20">
-        <f>IF(L38&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L38)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L38)),"")</f>
+        <f>IF(L38&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L38,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L38,23)),"")</f>
         <v/>
       </c>
       <c r="O38" s="20">
-        <f>IF(L38&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L38)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L38)),"")</f>
+        <f>IF(L38&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L38,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L38,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P38" s="20">
+        <f>IF(L38&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L38,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L38,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="39" hidden="1" ht="26" customHeight="1">
       <c r="A39" s="15">
-        <f>IF(L39&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L39),"")</f>
+        <f>IF(OR(J39=0,K39=1),"",COUNTIF(K$15:K39,0)-COUNTIF(J$15:J39,0))</f>
         <v/>
       </c>
       <c r="B39" s="15" t="n"/>
       <c r="C39" s="16">
-        <f>IF(J39=0,"",IF(K39=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J39)),IF(L39&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L39),INDEX('2 Import devis'!$B$6:$B$29,J39))))</f>
+        <f>IF(J39=0,"",IF(K39=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J39)),IF(L39&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L39,2)),INDEX('2 Import devis'!$B$6:$B$29,J39))))</f>
         <v/>
       </c>
       <c r="D39" s="17">
@@ -2458,11 +2569,11 @@
         <v/>
       </c>
       <c r="E39" s="17">
-        <f>IF(K39=1,"",IF(L39&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L39)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L39)),"FR"))</f>
+        <f>IF(OR(J39=0,K39=1),"",IF(L39&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L39,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L39,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L39,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F39" s="18">
-        <f>IF(L39&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L39)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L39)),"")</f>
+        <f>IF(L39&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L39,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L39,3),1)),"")</f>
         <v/>
       </c>
       <c r="G39" s="19">
@@ -2486,26 +2597,30 @@
         <v/>
       </c>
       <c r="M39" s="20">
-        <f>IF(L39&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L39)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L39)),"")</f>
+        <f>IF(L39&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L39,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L39,20)),"")</f>
         <v/>
       </c>
       <c r="N39" s="20">
-        <f>IF(L39&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L39)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L39)),"")</f>
+        <f>IF(L39&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L39,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L39,23)),"")</f>
         <v/>
       </c>
       <c r="O39" s="20">
-        <f>IF(L39&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L39)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L39)),"")</f>
+        <f>IF(L39&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L39,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L39,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P39" s="20">
+        <f>IF(L39&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L39,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L39,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="40" hidden="1" ht="26" customHeight="1">
       <c r="A40" s="15">
-        <f>IF(L40&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L40),"")</f>
+        <f>IF(OR(J40=0,K40=1),"",COUNTIF(K$15:K40,0)-COUNTIF(J$15:J40,0))</f>
         <v/>
       </c>
       <c r="B40" s="15" t="n"/>
       <c r="C40" s="16">
-        <f>IF(J40=0,"",IF(K40=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J40)),IF(L40&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L40),INDEX('2 Import devis'!$B$6:$B$29,J40))))</f>
+        <f>IF(J40=0,"",IF(K40=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J40)),IF(L40&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L40,2)),INDEX('2 Import devis'!$B$6:$B$29,J40))))</f>
         <v/>
       </c>
       <c r="D40" s="17">
@@ -2513,11 +2628,11 @@
         <v/>
       </c>
       <c r="E40" s="17">
-        <f>IF(K40=1,"",IF(L40&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L40)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L40)),"FR"))</f>
+        <f>IF(OR(J40=0,K40=1),"",IF(L40&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L40,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L40,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L40,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F40" s="18">
-        <f>IF(L40&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L40)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L40)),"")</f>
+        <f>IF(L40&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L40,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L40,3),1)),"")</f>
         <v/>
       </c>
       <c r="G40" s="19">
@@ -2541,26 +2656,30 @@
         <v/>
       </c>
       <c r="M40" s="20">
-        <f>IF(L40&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L40)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L40)),"")</f>
+        <f>IF(L40&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L40,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L40,20)),"")</f>
         <v/>
       </c>
       <c r="N40" s="20">
-        <f>IF(L40&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L40)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L40)),"")</f>
+        <f>IF(L40&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L40,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L40,23)),"")</f>
         <v/>
       </c>
       <c r="O40" s="20">
-        <f>IF(L40&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L40)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L40)),"")</f>
+        <f>IF(L40&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L40,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L40,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P40" s="20">
+        <f>IF(L40&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L40,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L40,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="41" hidden="1" ht="26" customHeight="1">
       <c r="A41" s="15">
-        <f>IF(L41&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L41),"")</f>
+        <f>IF(OR(J41=0,K41=1),"",COUNTIF(K$15:K41,0)-COUNTIF(J$15:J41,0))</f>
         <v/>
       </c>
       <c r="B41" s="15" t="n"/>
       <c r="C41" s="16">
-        <f>IF(J41=0,"",IF(K41=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J41)),IF(L41&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L41),INDEX('2 Import devis'!$B$6:$B$29,J41))))</f>
+        <f>IF(J41=0,"",IF(K41=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J41)),IF(L41&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L41,2)),INDEX('2 Import devis'!$B$6:$B$29,J41))))</f>
         <v/>
       </c>
       <c r="D41" s="17">
@@ -2568,11 +2687,11 @@
         <v/>
       </c>
       <c r="E41" s="17">
-        <f>IF(K41=1,"",IF(L41&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L41)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L41)),"FR"))</f>
+        <f>IF(OR(J41=0,K41=1),"",IF(L41&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L41,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L41,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L41,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F41" s="18">
-        <f>IF(L41&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L41)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L41)),"")</f>
+        <f>IF(L41&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L41,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L41,3),1)),"")</f>
         <v/>
       </c>
       <c r="G41" s="19">
@@ -2596,26 +2715,30 @@
         <v/>
       </c>
       <c r="M41" s="20">
-        <f>IF(L41&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L41)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L41)),"")</f>
+        <f>IF(L41&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L41,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L41,20)),"")</f>
         <v/>
       </c>
       <c r="N41" s="20">
-        <f>IF(L41&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L41)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L41)),"")</f>
+        <f>IF(L41&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L41,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L41,23)),"")</f>
         <v/>
       </c>
       <c r="O41" s="20">
-        <f>IF(L41&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L41)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L41)),"")</f>
+        <f>IF(L41&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L41,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L41,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P41" s="20">
+        <f>IF(L41&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L41,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L41,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="42" hidden="1" ht="26" customHeight="1">
       <c r="A42" s="15">
-        <f>IF(L42&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L42),"")</f>
+        <f>IF(OR(J42=0,K42=1),"",COUNTIF(K$15:K42,0)-COUNTIF(J$15:J42,0))</f>
         <v/>
       </c>
       <c r="B42" s="15" t="n"/>
       <c r="C42" s="16">
-        <f>IF(J42=0,"",IF(K42=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J42)),IF(L42&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L42),INDEX('2 Import devis'!$B$6:$B$29,J42))))</f>
+        <f>IF(J42=0,"",IF(K42=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J42)),IF(L42&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L42,2)),INDEX('2 Import devis'!$B$6:$B$29,J42))))</f>
         <v/>
       </c>
       <c r="D42" s="17">
@@ -2623,11 +2746,11 @@
         <v/>
       </c>
       <c r="E42" s="17">
-        <f>IF(K42=1,"",IF(L42&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L42)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L42)),"FR"))</f>
+        <f>IF(OR(J42=0,K42=1),"",IF(L42&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L42,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L42,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L42,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F42" s="18">
-        <f>IF(L42&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L42)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L42)),"")</f>
+        <f>IF(L42&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L42,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L42,3),1)),"")</f>
         <v/>
       </c>
       <c r="G42" s="19">
@@ -2651,26 +2774,30 @@
         <v/>
       </c>
       <c r="M42" s="20">
-        <f>IF(L42&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L42)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L42)),"")</f>
+        <f>IF(L42&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L42,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L42,20)),"")</f>
         <v/>
       </c>
       <c r="N42" s="20">
-        <f>IF(L42&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L42)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L42)),"")</f>
+        <f>IF(L42&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L42,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L42,23)),"")</f>
         <v/>
       </c>
       <c r="O42" s="20">
-        <f>IF(L42&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L42)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L42)),"")</f>
+        <f>IF(L42&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L42,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L42,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P42" s="20">
+        <f>IF(L42&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L42,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L42,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="43" hidden="1" ht="26" customHeight="1">
       <c r="A43" s="15">
-        <f>IF(L43&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L43),"")</f>
+        <f>IF(OR(J43=0,K43=1),"",COUNTIF(K$15:K43,0)-COUNTIF(J$15:J43,0))</f>
         <v/>
       </c>
       <c r="B43" s="15" t="n"/>
       <c r="C43" s="16">
-        <f>IF(J43=0,"",IF(K43=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J43)),IF(L43&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L43),INDEX('2 Import devis'!$B$6:$B$29,J43))))</f>
+        <f>IF(J43=0,"",IF(K43=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J43)),IF(L43&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L43,2)),INDEX('2 Import devis'!$B$6:$B$29,J43))))</f>
         <v/>
       </c>
       <c r="D43" s="17">
@@ -2678,11 +2805,11 @@
         <v/>
       </c>
       <c r="E43" s="17">
-        <f>IF(K43=1,"",IF(L43&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L43)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L43)),"FR"))</f>
+        <f>IF(OR(J43=0,K43=1),"",IF(L43&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L43,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L43,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L43,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F43" s="18">
-        <f>IF(L43&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L43)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L43)),"")</f>
+        <f>IF(L43&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L43,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L43,3),1)),"")</f>
         <v/>
       </c>
       <c r="G43" s="19">
@@ -2706,26 +2833,30 @@
         <v/>
       </c>
       <c r="M43" s="20">
-        <f>IF(L43&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L43)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L43)),"")</f>
+        <f>IF(L43&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L43,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L43,20)),"")</f>
         <v/>
       </c>
       <c r="N43" s="20">
-        <f>IF(L43&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L43)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L43)),"")</f>
+        <f>IF(L43&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L43,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L43,23)),"")</f>
         <v/>
       </c>
       <c r="O43" s="20">
-        <f>IF(L43&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L43)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L43)),"")</f>
+        <f>IF(L43&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L43,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L43,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P43" s="20">
+        <f>IF(L43&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L43,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L43,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="44" hidden="1" ht="26" customHeight="1">
       <c r="A44" s="15">
-        <f>IF(L44&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L44),"")</f>
+        <f>IF(OR(J44=0,K44=1),"",COUNTIF(K$15:K44,0)-COUNTIF(J$15:J44,0))</f>
         <v/>
       </c>
       <c r="B44" s="15" t="n"/>
       <c r="C44" s="16">
-        <f>IF(J44=0,"",IF(K44=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J44)),IF(L44&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L44),INDEX('2 Import devis'!$B$6:$B$29,J44))))</f>
+        <f>IF(J44=0,"",IF(K44=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J44)),IF(L44&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L44,2)),INDEX('2 Import devis'!$B$6:$B$29,J44))))</f>
         <v/>
       </c>
       <c r="D44" s="17">
@@ -2733,11 +2864,11 @@
         <v/>
       </c>
       <c r="E44" s="17">
-        <f>IF(K44=1,"",IF(L44&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L44)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L44)),"FR"))</f>
+        <f>IF(OR(J44=0,K44=1),"",IF(L44&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L44,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L44,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L44,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F44" s="18">
-        <f>IF(L44&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L44)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L44)),"")</f>
+        <f>IF(L44&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L44,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L44,3),1)),"")</f>
         <v/>
       </c>
       <c r="G44" s="19">
@@ -2761,26 +2892,30 @@
         <v/>
       </c>
       <c r="M44" s="20">
-        <f>IF(L44&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L44)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L44)),"")</f>
+        <f>IF(L44&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L44,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L44,20)),"")</f>
         <v/>
       </c>
       <c r="N44" s="20">
-        <f>IF(L44&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L44)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L44)),"")</f>
+        <f>IF(L44&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L44,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L44,23)),"")</f>
         <v/>
       </c>
       <c r="O44" s="20">
-        <f>IF(L44&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L44)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L44)),"")</f>
+        <f>IF(L44&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L44,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L44,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P44" s="20">
+        <f>IF(L44&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L44,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L44,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="45" hidden="1" ht="26" customHeight="1">
       <c r="A45" s="15">
-        <f>IF(L45&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L45),"")</f>
+        <f>IF(OR(J45=0,K45=1),"",COUNTIF(K$15:K45,0)-COUNTIF(J$15:J45,0))</f>
         <v/>
       </c>
       <c r="B45" s="15" t="n"/>
       <c r="C45" s="16">
-        <f>IF(J45=0,"",IF(K45=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J45)),IF(L45&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L45),INDEX('2 Import devis'!$B$6:$B$29,J45))))</f>
+        <f>IF(J45=0,"",IF(K45=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J45)),IF(L45&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L45,2)),INDEX('2 Import devis'!$B$6:$B$29,J45))))</f>
         <v/>
       </c>
       <c r="D45" s="17">
@@ -2788,11 +2923,11 @@
         <v/>
       </c>
       <c r="E45" s="17">
-        <f>IF(K45=1,"",IF(L45&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L45)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L45)),"FR"))</f>
+        <f>IF(OR(J45=0,K45=1),"",IF(L45&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L45,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L45,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L45,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F45" s="18">
-        <f>IF(L45&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L45)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L45)),"")</f>
+        <f>IF(L45&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L45,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L45,3),1)),"")</f>
         <v/>
       </c>
       <c r="G45" s="19">
@@ -2816,26 +2951,30 @@
         <v/>
       </c>
       <c r="M45" s="20">
-        <f>IF(L45&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L45)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L45)),"")</f>
+        <f>IF(L45&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L45,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L45,20)),"")</f>
         <v/>
       </c>
       <c r="N45" s="20">
-        <f>IF(L45&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L45)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L45)),"")</f>
+        <f>IF(L45&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L45,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L45,23)),"")</f>
         <v/>
       </c>
       <c r="O45" s="20">
-        <f>IF(L45&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L45)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L45)),"")</f>
+        <f>IF(L45&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L45,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L45,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P45" s="20">
+        <f>IF(L45&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L45,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L45,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="46" hidden="1" ht="26" customHeight="1">
       <c r="A46" s="15">
-        <f>IF(L46&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L46),"")</f>
+        <f>IF(OR(J46=0,K46=1),"",COUNTIF(K$15:K46,0)-COUNTIF(J$15:J46,0))</f>
         <v/>
       </c>
       <c r="B46" s="15" t="n"/>
       <c r="C46" s="16">
-        <f>IF(J46=0,"",IF(K46=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J46)),IF(L46&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L46),INDEX('2 Import devis'!$B$6:$B$29,J46))))</f>
+        <f>IF(J46=0,"",IF(K46=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J46)),IF(L46&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L46,2)),INDEX('2 Import devis'!$B$6:$B$29,J46))))</f>
         <v/>
       </c>
       <c r="D46" s="17">
@@ -2843,11 +2982,11 @@
         <v/>
       </c>
       <c r="E46" s="17">
-        <f>IF(K46=1,"",IF(L46&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L46)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L46)),"FR"))</f>
+        <f>IF(OR(J46=0,K46=1),"",IF(L46&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L46,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L46,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L46,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F46" s="18">
-        <f>IF(L46&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L46)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L46)),"")</f>
+        <f>IF(L46&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L46,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L46,3),1)),"")</f>
         <v/>
       </c>
       <c r="G46" s="19">
@@ -2871,26 +3010,30 @@
         <v/>
       </c>
       <c r="M46" s="20">
-        <f>IF(L46&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L46)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L46)),"")</f>
+        <f>IF(L46&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L46,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L46,20)),"")</f>
         <v/>
       </c>
       <c r="N46" s="20">
-        <f>IF(L46&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L46)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L46)),"")</f>
+        <f>IF(L46&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L46,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L46,23)),"")</f>
         <v/>
       </c>
       <c r="O46" s="20">
-        <f>IF(L46&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L46)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L46)),"")</f>
+        <f>IF(L46&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L46,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L46,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P46" s="20">
+        <f>IF(L46&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L46,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L46,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="47" hidden="1" ht="26" customHeight="1">
       <c r="A47" s="15">
-        <f>IF(L47&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L47),"")</f>
+        <f>IF(OR(J47=0,K47=1),"",COUNTIF(K$15:K47,0)-COUNTIF(J$15:J47,0))</f>
         <v/>
       </c>
       <c r="B47" s="15" t="n"/>
       <c r="C47" s="16">
-        <f>IF(J47=0,"",IF(K47=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J47)),IF(L47&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L47),INDEX('2 Import devis'!$B$6:$B$29,J47))))</f>
+        <f>IF(J47=0,"",IF(K47=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J47)),IF(L47&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L47,2)),INDEX('2 Import devis'!$B$6:$B$29,J47))))</f>
         <v/>
       </c>
       <c r="D47" s="17">
@@ -2898,11 +3041,11 @@
         <v/>
       </c>
       <c r="E47" s="17">
-        <f>IF(K47=1,"",IF(L47&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L47)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L47)),"FR"))</f>
+        <f>IF(OR(J47=0,K47=1),"",IF(L47&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L47,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L47,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L47,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F47" s="18">
-        <f>IF(L47&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L47)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L47)),"")</f>
+        <f>IF(L47&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L47,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L47,3),1)),"")</f>
         <v/>
       </c>
       <c r="G47" s="19">
@@ -2926,26 +3069,30 @@
         <v/>
       </c>
       <c r="M47" s="20">
-        <f>IF(L47&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L47)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L47)),"")</f>
+        <f>IF(L47&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L47,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L47,20)),"")</f>
         <v/>
       </c>
       <c r="N47" s="20">
-        <f>IF(L47&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L47)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L47)),"")</f>
+        <f>IF(L47&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L47,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L47,23)),"")</f>
         <v/>
       </c>
       <c r="O47" s="20">
-        <f>IF(L47&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L47)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L47)),"")</f>
+        <f>IF(L47&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L47,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L47,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P47" s="20">
+        <f>IF(L47&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L47,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L47,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="48" hidden="1" ht="26" customHeight="1">
       <c r="A48" s="15">
-        <f>IF(L48&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L48),"")</f>
+        <f>IF(OR(J48=0,K48=1),"",COUNTIF(K$15:K48,0)-COUNTIF(J$15:J48,0))</f>
         <v/>
       </c>
       <c r="B48" s="15" t="n"/>
       <c r="C48" s="16">
-        <f>IF(J48=0,"",IF(K48=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J48)),IF(L48&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L48),INDEX('2 Import devis'!$B$6:$B$29,J48))))</f>
+        <f>IF(J48=0,"",IF(K48=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J48)),IF(L48&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L48,2)),INDEX('2 Import devis'!$B$6:$B$29,J48))))</f>
         <v/>
       </c>
       <c r="D48" s="17">
@@ -2953,11 +3100,11 @@
         <v/>
       </c>
       <c r="E48" s="17">
-        <f>IF(K48=1,"",IF(L48&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L48)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L48)),"FR"))</f>
+        <f>IF(OR(J48=0,K48=1),"",IF(L48&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L48,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L48,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L48,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F48" s="18">
-        <f>IF(L48&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L48)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L48)),"")</f>
+        <f>IF(L48&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L48,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L48,3),1)),"")</f>
         <v/>
       </c>
       <c r="G48" s="19">
@@ -2981,26 +3128,30 @@
         <v/>
       </c>
       <c r="M48" s="20">
-        <f>IF(L48&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L48)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L48)),"")</f>
+        <f>IF(L48&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L48,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L48,20)),"")</f>
         <v/>
       </c>
       <c r="N48" s="20">
-        <f>IF(L48&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L48)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L48)),"")</f>
+        <f>IF(L48&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L48,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L48,23)),"")</f>
         <v/>
       </c>
       <c r="O48" s="20">
-        <f>IF(L48&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L48)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L48)),"")</f>
+        <f>IF(L48&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L48,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L48,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P48" s="20">
+        <f>IF(L48&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L48,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L48,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="49" hidden="1" ht="26" customHeight="1">
       <c r="A49" s="15">
-        <f>IF(L49&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L49),"")</f>
+        <f>IF(OR(J49=0,K49=1),"",COUNTIF(K$15:K49,0)-COUNTIF(J$15:J49,0))</f>
         <v/>
       </c>
       <c r="B49" s="15" t="n"/>
       <c r="C49" s="16">
-        <f>IF(J49=0,"",IF(K49=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J49)),IF(L49&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L49),INDEX('2 Import devis'!$B$6:$B$29,J49))))</f>
+        <f>IF(J49=0,"",IF(K49=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J49)),IF(L49&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L49,2)),INDEX('2 Import devis'!$B$6:$B$29,J49))))</f>
         <v/>
       </c>
       <c r="D49" s="17">
@@ -3008,11 +3159,11 @@
         <v/>
       </c>
       <c r="E49" s="17">
-        <f>IF(K49=1,"",IF(L49&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L49)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L49)),"FR"))</f>
+        <f>IF(OR(J49=0,K49=1),"",IF(L49&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L49,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L49,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L49,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F49" s="18">
-        <f>IF(L49&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L49)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L49)),"")</f>
+        <f>IF(L49&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L49,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L49,3),1)),"")</f>
         <v/>
       </c>
       <c r="G49" s="19">
@@ -3036,26 +3187,30 @@
         <v/>
       </c>
       <c r="M49" s="20">
-        <f>IF(L49&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L49)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L49)),"")</f>
+        <f>IF(L49&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L49,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L49,20)),"")</f>
         <v/>
       </c>
       <c r="N49" s="20">
-        <f>IF(L49&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L49)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L49)),"")</f>
+        <f>IF(L49&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L49,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L49,23)),"")</f>
         <v/>
       </c>
       <c r="O49" s="20">
-        <f>IF(L49&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L49)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L49)),"")</f>
+        <f>IF(L49&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L49,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L49,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P49" s="20">
+        <f>IF(L49&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L49,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L49,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="50" hidden="1" ht="26" customHeight="1">
       <c r="A50" s="15">
-        <f>IF(L50&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L50),"")</f>
+        <f>IF(OR(J50=0,K50=1),"",COUNTIF(K$15:K50,0)-COUNTIF(J$15:J50,0))</f>
         <v/>
       </c>
       <c r="B50" s="15" t="n"/>
       <c r="C50" s="16">
-        <f>IF(J50=0,"",IF(K50=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J50)),IF(L50&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L50),INDEX('2 Import devis'!$B$6:$B$29,J50))))</f>
+        <f>IF(J50=0,"",IF(K50=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J50)),IF(L50&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L50,2)),INDEX('2 Import devis'!$B$6:$B$29,J50))))</f>
         <v/>
       </c>
       <c r="D50" s="17">
@@ -3063,11 +3218,11 @@
         <v/>
       </c>
       <c r="E50" s="17">
-        <f>IF(K50=1,"",IF(L50&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L50)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L50)),"FR"))</f>
+        <f>IF(OR(J50=0,K50=1),"",IF(L50&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L50,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L50,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L50,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F50" s="18">
-        <f>IF(L50&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L50)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L50)),"")</f>
+        <f>IF(L50&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L50,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L50,3),1)),"")</f>
         <v/>
       </c>
       <c r="G50" s="19">
@@ -3091,26 +3246,30 @@
         <v/>
       </c>
       <c r="M50" s="20">
-        <f>IF(L50&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L50)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L50)),"")</f>
+        <f>IF(L50&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L50,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L50,20)),"")</f>
         <v/>
       </c>
       <c r="N50" s="20">
-        <f>IF(L50&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L50)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L50)),"")</f>
+        <f>IF(L50&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L50,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L50,23)),"")</f>
         <v/>
       </c>
       <c r="O50" s="20">
-        <f>IF(L50&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L50)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L50)),"")</f>
+        <f>IF(L50&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L50,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L50,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P50" s="20">
+        <f>IF(L50&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L50,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L50,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="51" hidden="1" ht="26" customHeight="1">
       <c r="A51" s="15">
-        <f>IF(L51&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L51),"")</f>
+        <f>IF(OR(J51=0,K51=1),"",COUNTIF(K$15:K51,0)-COUNTIF(J$15:J51,0))</f>
         <v/>
       </c>
       <c r="B51" s="15" t="n"/>
       <c r="C51" s="16">
-        <f>IF(J51=0,"",IF(K51=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J51)),IF(L51&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L51),INDEX('2 Import devis'!$B$6:$B$29,J51))))</f>
+        <f>IF(J51=0,"",IF(K51=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J51)),IF(L51&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L51,2)),INDEX('2 Import devis'!$B$6:$B$29,J51))))</f>
         <v/>
       </c>
       <c r="D51" s="17">
@@ -3118,11 +3277,11 @@
         <v/>
       </c>
       <c r="E51" s="17">
-        <f>IF(K51=1,"",IF(L51&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L51)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L51)),"FR"))</f>
+        <f>IF(OR(J51=0,K51=1),"",IF(L51&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L51,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L51,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L51,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F51" s="18">
-        <f>IF(L51&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L51)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L51)),"")</f>
+        <f>IF(L51&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L51,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L51,3),1)),"")</f>
         <v/>
       </c>
       <c r="G51" s="19">
@@ -3146,26 +3305,30 @@
         <v/>
       </c>
       <c r="M51" s="20">
-        <f>IF(L51&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L51)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L51)),"")</f>
+        <f>IF(L51&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L51,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L51,20)),"")</f>
         <v/>
       </c>
       <c r="N51" s="20">
-        <f>IF(L51&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L51)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L51)),"")</f>
+        <f>IF(L51&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L51,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L51,23)),"")</f>
         <v/>
       </c>
       <c r="O51" s="20">
-        <f>IF(L51&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L51)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L51)),"")</f>
+        <f>IF(L51&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L51,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L51,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P51" s="20">
+        <f>IF(L51&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L51,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L51,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="52" hidden="1" ht="26" customHeight="1">
       <c r="A52" s="15">
-        <f>IF(L52&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L52),"")</f>
+        <f>IF(OR(J52=0,K52=1),"",COUNTIF(K$15:K52,0)-COUNTIF(J$15:J52,0))</f>
         <v/>
       </c>
       <c r="B52" s="15" t="n"/>
       <c r="C52" s="16">
-        <f>IF(J52=0,"",IF(K52=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J52)),IF(L52&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L52),INDEX('2 Import devis'!$B$6:$B$29,J52))))</f>
+        <f>IF(J52=0,"",IF(K52=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J52)),IF(L52&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L52,2)),INDEX('2 Import devis'!$B$6:$B$29,J52))))</f>
         <v/>
       </c>
       <c r="D52" s="17">
@@ -3173,11 +3336,11 @@
         <v/>
       </c>
       <c r="E52" s="17">
-        <f>IF(K52=1,"",IF(L52&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L52)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L52)),"FR"))</f>
+        <f>IF(OR(J52=0,K52=1),"",IF(L52&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L52,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L52,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L52,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F52" s="18">
-        <f>IF(L52&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L52)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L52)),"")</f>
+        <f>IF(L52&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L52,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L52,3),1)),"")</f>
         <v/>
       </c>
       <c r="G52" s="19">
@@ -3201,26 +3364,30 @@
         <v/>
       </c>
       <c r="M52" s="20">
-        <f>IF(L52&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L52)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L52)),"")</f>
+        <f>IF(L52&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L52,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L52,20)),"")</f>
         <v/>
       </c>
       <c r="N52" s="20">
-        <f>IF(L52&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L52)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L52)),"")</f>
+        <f>IF(L52&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L52,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L52,23)),"")</f>
         <v/>
       </c>
       <c r="O52" s="20">
-        <f>IF(L52&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L52)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L52)),"")</f>
+        <f>IF(L52&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L52,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L52,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P52" s="20">
+        <f>IF(L52&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L52,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L52,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="53" hidden="1" ht="26" customHeight="1">
       <c r="A53" s="15">
-        <f>IF(L53&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L53),"")</f>
+        <f>IF(OR(J53=0,K53=1),"",COUNTIF(K$15:K53,0)-COUNTIF(J$15:J53,0))</f>
         <v/>
       </c>
       <c r="B53" s="15" t="n"/>
       <c r="C53" s="16">
-        <f>IF(J53=0,"",IF(K53=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J53)),IF(L53&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L53),INDEX('2 Import devis'!$B$6:$B$29,J53))))</f>
+        <f>IF(J53=0,"",IF(K53=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J53)),IF(L53&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L53,2)),INDEX('2 Import devis'!$B$6:$B$29,J53))))</f>
         <v/>
       </c>
       <c r="D53" s="17">
@@ -3228,11 +3395,11 @@
         <v/>
       </c>
       <c r="E53" s="17">
-        <f>IF(K53=1,"",IF(L53&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L53)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L53)),"FR"))</f>
+        <f>IF(OR(J53=0,K53=1),"",IF(L53&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L53,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L53,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L53,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F53" s="18">
-        <f>IF(L53&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L53)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L53)),"")</f>
+        <f>IF(L53&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L53,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L53,3),1)),"")</f>
         <v/>
       </c>
       <c r="G53" s="19">
@@ -3256,26 +3423,30 @@
         <v/>
       </c>
       <c r="M53" s="20">
-        <f>IF(L53&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L53)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L53)),"")</f>
+        <f>IF(L53&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L53,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L53,20)),"")</f>
         <v/>
       </c>
       <c r="N53" s="20">
-        <f>IF(L53&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L53)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L53)),"")</f>
+        <f>IF(L53&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L53,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L53,23)),"")</f>
         <v/>
       </c>
       <c r="O53" s="20">
-        <f>IF(L53&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L53)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L53)),"")</f>
+        <f>IF(L53&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L53,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L53,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P53" s="20">
+        <f>IF(L53&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L53,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L53,5)),"")</f>
         <v/>
       </c>
     </row>
     <row r="54" hidden="1" ht="26" customHeight="1">
       <c r="A54" s="15">
-        <f>IF(L54&gt;0,INDEX('3 Catalogue outils'!$B$6:$B$5005,L54),"")</f>
+        <f>IF(OR(J54=0,K54=1),"",COUNTIF(K$15:K54,0)-COUNTIF(J$15:J54,0))</f>
         <v/>
       </c>
       <c r="B54" s="15" t="n"/>
       <c r="C54" s="16">
-        <f>IF(J54=0,"",IF(K54=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J54)),IF(L54&gt;0,INDEX('3 Catalogue outils'!$C$6:$C$5005,L54),INDEX('2 Import devis'!$B$6:$B$29,J54))))</f>
+        <f>IF(J54=0,"",IF(K54=1,UPPER(INDEX('2 Import devis'!$B$6:$B$29,J54)),IF(L54&gt;0,CLEAN(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L54,2)),INDEX('2 Import devis'!$B$6:$B$29,J54))))</f>
         <v/>
       </c>
       <c r="D54" s="17">
@@ -3283,11 +3454,11 @@
         <v/>
       </c>
       <c r="E54" s="17">
-        <f>IF(K54=1,"",IF(L54&gt;0,IF(INDEX('3 Catalogue outils'!$D$6:$D$5005,L54)="","FR",INDEX('3 Catalogue outils'!$D$6:$D$5005,L54)),"FR"))</f>
+        <f>IF(OR(J54=0,K54=1),"",IF(L54&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L54,22))=0,IF(ISTEXT(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L54,22)),INDEX('3 Catalogue outils'!$A$6:$AC$5005,L54,22),"FR"),"FR"),"FR"))</f>
         <v/>
       </c>
       <c r="F54" s="18">
-        <f>IF(L54&gt;0,IF(INDEX('3 Catalogue outils'!$F$6:$F$5005,L54)="","",INDEX('3 Catalogue outils'!$F$6:$F$5005,L54)),"")</f>
+        <f>IF(L54&gt;0,IF(N(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L54,3))=0,"",ROUND(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L54,3),1)),"")</f>
         <v/>
       </c>
       <c r="G54" s="19">
@@ -3311,15 +3482,19 @@
         <v/>
       </c>
       <c r="M54" s="20">
-        <f>IF(L54&gt;0,IF(INDEX('3 Catalogue outils'!$E$6:$E$5005,L54)="","",INDEX('3 Catalogue outils'!$E$6:$E$5005,L54)),"")</f>
+        <f>IF(L54&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L54,20)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L54,20)),"")</f>
         <v/>
       </c>
       <c r="N54" s="20">
-        <f>IF(L54&gt;0,IF(INDEX('3 Catalogue outils'!$G$6:$G$5005,L54)="","",INDEX('3 Catalogue outils'!$G$6:$G$5005,L54)),"")</f>
+        <f>IF(L54&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L54,23)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L54,23)),"")</f>
         <v/>
       </c>
       <c r="O54" s="20">
-        <f>IF(L54&gt;0,IF(INDEX('3 Catalogue outils'!$H$6:$H$5005,L54)="","",INDEX('3 Catalogue outils'!$H$6:$H$5005,L54)),"")</f>
+        <f>IF(L54&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L54,4)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L54,4)),"")</f>
+        <v/>
+      </c>
+      <c r="P54" s="20">
+        <f>IF(L54&gt;0,IF(INDEX('3 Catalogue outils'!$A$6:$AC$5005,L54,5)=0,"",INDEX('3 Catalogue outils'!$A$6:$AC$5005,L54,5)),"")</f>
         <v/>
       </c>
     </row>
@@ -4154,17 +4329,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H65"/>
+  <dimension ref="A1:AC65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="56" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="7" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="7" customWidth="1" min="16" max="16"/>
+    <col width="7" customWidth="1" min="17" max="17"/>
+    <col width="7" customWidth="1" min="18" max="18"/>
+    <col width="7" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="7" customWidth="1" min="21" max="21"/>
+    <col width="10" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="7" customWidth="1" min="24" max="24"/>
+    <col width="7" customWidth="1" min="25" max="25"/>
+    <col width="7" customWidth="1" min="26" max="26"/>
+    <col width="7" customWidth="1" min="27" max="27"/>
+    <col width="7" customWidth="1" min="28" max="28"/>
+    <col width="7" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -4180,11 +4376,32 @@
       <c r="F1" s="1" t="n"/>
       <c r="G1" s="1" t="n"/>
       <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
+      <c r="J1" s="1" t="n"/>
+      <c r="K1" s="1" t="n"/>
+      <c r="L1" s="1" t="n"/>
+      <c r="M1" s="1" t="n"/>
+      <c r="N1" s="1" t="n"/>
+      <c r="O1" s="1" t="n"/>
+      <c r="P1" s="1" t="n"/>
+      <c r="Q1" s="1" t="n"/>
+      <c r="R1" s="1" t="n"/>
+      <c r="S1" s="1" t="n"/>
+      <c r="T1" s="1" t="n"/>
+      <c r="U1" s="1" t="n"/>
+      <c r="V1" s="1" t="n"/>
+      <c r="W1" s="1" t="n"/>
+      <c r="X1" s="1" t="n"/>
+      <c r="Y1" s="1" t="n"/>
+      <c r="Z1" s="1" t="n"/>
+      <c r="AA1" s="1" t="n"/>
+      <c r="AB1" s="1" t="n"/>
+      <c r="AC1" s="1" t="n"/>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="56" t="inlineStr">
         <is>
-          <t>Coller ici votre registre des outils (en-têtes ligne 5, données dès la ligne 6). Le BL retrouve référence, désignation, origine et poids à partir du N° de série saisi en colonne B du BL.</t>
+          <t>Dans le registre « Fabrication - Achat - 2014 et + » : copier les colonnes Z à BB (à partir de la ligne 2) et les coller ici en A6. Le BL cherche le N° de série (colonne A) et reprend désignation, poids, référence, origine, code SH, OD et longueur.</t>
         </is>
       </c>
       <c r="B2" s="1" t="n"/>
@@ -4194,6 +4411,27 @@
       <c r="F2" s="1" t="n"/>
       <c r="G2" s="1" t="n"/>
       <c r="H2" s="1" t="n"/>
+      <c r="I2" s="1" t="n"/>
+      <c r="J2" s="1" t="n"/>
+      <c r="K2" s="1" t="n"/>
+      <c r="L2" s="1" t="n"/>
+      <c r="M2" s="1" t="n"/>
+      <c r="N2" s="1" t="n"/>
+      <c r="O2" s="1" t="n"/>
+      <c r="P2" s="1" t="n"/>
+      <c r="Q2" s="1" t="n"/>
+      <c r="R2" s="1" t="n"/>
+      <c r="S2" s="1" t="n"/>
+      <c r="T2" s="1" t="n"/>
+      <c r="U2" s="1" t="n"/>
+      <c r="V2" s="1" t="n"/>
+      <c r="W2" s="1" t="n"/>
+      <c r="X2" s="1" t="n"/>
+      <c r="Y2" s="1" t="n"/>
+      <c r="Z2" s="1" t="n"/>
+      <c r="AA2" s="1" t="n"/>
+      <c r="AB2" s="1" t="n"/>
+      <c r="AC2" s="1" t="n"/>
     </row>
     <row r="3" ht="5" customHeight="1">
       <c r="A3" s="57" t="n"/>
@@ -4204,6 +4442,27 @@
       <c r="F3" s="57" t="n"/>
       <c r="G3" s="57" t="n"/>
       <c r="H3" s="57" t="n"/>
+      <c r="I3" s="57" t="n"/>
+      <c r="J3" s="57" t="n"/>
+      <c r="K3" s="57" t="n"/>
+      <c r="L3" s="57" t="n"/>
+      <c r="M3" s="57" t="n"/>
+      <c r="N3" s="57" t="n"/>
+      <c r="O3" s="57" t="n"/>
+      <c r="P3" s="57" t="n"/>
+      <c r="Q3" s="57" t="n"/>
+      <c r="R3" s="57" t="n"/>
+      <c r="S3" s="57" t="n"/>
+      <c r="T3" s="57" t="n"/>
+      <c r="U3" s="57" t="n"/>
+      <c r="V3" s="57" t="n"/>
+      <c r="W3" s="57" t="n"/>
+      <c r="X3" s="57" t="n"/>
+      <c r="Y3" s="57" t="n"/>
+      <c r="Z3" s="57" t="n"/>
+      <c r="AA3" s="57" t="n"/>
+      <c r="AB3" s="57" t="n"/>
+      <c r="AC3" s="57" t="n"/>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="50" t="inlineStr">
@@ -4213,639 +4472,2004 @@
       </c>
       <c r="B5" s="50" t="inlineStr">
         <is>
+          <t>Désignation</t>
+        </is>
+      </c>
+      <c r="C5" s="50" t="inlineStr">
+        <is>
+          <t>Poids net (kg)</t>
+        </is>
+      </c>
+      <c r="D5" s="50" t="inlineStr">
+        <is>
+          <t>OD</t>
+        </is>
+      </c>
+      <c r="E5" s="50" t="inlineStr">
+        <is>
+          <t>Longueur (mm)</t>
+        </is>
+      </c>
+      <c r="F5" s="51" t="inlineStr">
+        <is>
+          <t>col. 6</t>
+        </is>
+      </c>
+      <c r="G5" s="51" t="inlineStr">
+        <is>
+          <t>col. 7</t>
+        </is>
+      </c>
+      <c r="H5" s="51" t="inlineStr">
+        <is>
+          <t>col. 8</t>
+        </is>
+      </c>
+      <c r="I5" s="51" t="inlineStr">
+        <is>
+          <t>col. 9</t>
+        </is>
+      </c>
+      <c r="J5" s="51" t="inlineStr">
+        <is>
+          <t>col. 10</t>
+        </is>
+      </c>
+      <c r="K5" s="51" t="inlineStr">
+        <is>
+          <t>col. 11</t>
+        </is>
+      </c>
+      <c r="L5" s="51" t="inlineStr">
+        <is>
+          <t>col. 12</t>
+        </is>
+      </c>
+      <c r="M5" s="51" t="inlineStr">
+        <is>
+          <t>col. 13</t>
+        </is>
+      </c>
+      <c r="N5" s="51" t="inlineStr">
+        <is>
+          <t>col. 14</t>
+        </is>
+      </c>
+      <c r="O5" s="51" t="inlineStr">
+        <is>
+          <t>col. 15</t>
+        </is>
+      </c>
+      <c r="P5" s="51" t="inlineStr">
+        <is>
+          <t>col. 16</t>
+        </is>
+      </c>
+      <c r="Q5" s="51" t="inlineStr">
+        <is>
+          <t>col. 17</t>
+        </is>
+      </c>
+      <c r="R5" s="51" t="inlineStr">
+        <is>
+          <t>col. 18</t>
+        </is>
+      </c>
+      <c r="S5" s="51" t="inlineStr">
+        <is>
+          <t>col. 19</t>
+        </is>
+      </c>
+      <c r="T5" s="50" t="inlineStr">
+        <is>
           <t>Référence</t>
         </is>
       </c>
-      <c r="C5" s="50" t="inlineStr">
-        <is>
-          <t>Désignation</t>
-        </is>
-      </c>
-      <c r="D5" s="50" t="inlineStr">
+      <c r="U5" s="51" t="inlineStr">
+        <is>
+          <t>col. 21</t>
+        </is>
+      </c>
+      <c r="V5" s="50" t="inlineStr">
         <is>
           <t>Origine</t>
         </is>
       </c>
-      <c r="E5" s="50" t="inlineStr">
+      <c r="W5" s="50" t="inlineStr">
         <is>
           <t>Code SH (HS)</t>
         </is>
       </c>
-      <c r="F5" s="50" t="inlineStr">
-        <is>
-          <t>Poids net (kg)</t>
-        </is>
-      </c>
-      <c r="G5" s="50" t="inlineStr">
-        <is>
-          <t>OD</t>
-        </is>
-      </c>
-      <c r="H5" s="50" t="inlineStr">
-        <is>
-          <t>Longueur</t>
+      <c r="X5" s="51" t="inlineStr">
+        <is>
+          <t>col. 24</t>
+        </is>
+      </c>
+      <c r="Y5" s="51" t="inlineStr">
+        <is>
+          <t>col. 25</t>
+        </is>
+      </c>
+      <c r="Z5" s="51" t="inlineStr">
+        <is>
+          <t>col. 26</t>
+        </is>
+      </c>
+      <c r="AA5" s="51" t="inlineStr">
+        <is>
+          <t>col. 27</t>
+        </is>
+      </c>
+      <c r="AB5" s="51" t="inlineStr">
+        <is>
+          <t>col. 28</t>
+        </is>
+      </c>
+      <c r="AC5" s="51" t="inlineStr">
+        <is>
+          <t>col. 29</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="53" t="n"/>
-      <c r="B6" s="53" t="n"/>
-      <c r="C6" s="52" t="n"/>
+      <c r="B6" s="52" t="n"/>
+      <c r="C6" s="53" t="n"/>
       <c r="D6" s="53" t="n"/>
       <c r="E6" s="53" t="n"/>
-      <c r="F6" s="53" t="n"/>
-      <c r="G6" s="53" t="n"/>
-      <c r="H6" s="53" t="n"/>
+      <c r="F6" s="58" t="n"/>
+      <c r="G6" s="58" t="n"/>
+      <c r="H6" s="58" t="n"/>
+      <c r="I6" s="58" t="n"/>
+      <c r="J6" s="58" t="n"/>
+      <c r="K6" s="58" t="n"/>
+      <c r="L6" s="58" t="n"/>
+      <c r="M6" s="58" t="n"/>
+      <c r="N6" s="58" t="n"/>
+      <c r="O6" s="58" t="n"/>
+      <c r="P6" s="58" t="n"/>
+      <c r="Q6" s="58" t="n"/>
+      <c r="R6" s="58" t="n"/>
+      <c r="S6" s="58" t="n"/>
+      <c r="T6" s="53" t="n"/>
+      <c r="U6" s="58" t="n"/>
+      <c r="V6" s="53" t="n"/>
+      <c r="W6" s="53" t="n"/>
+      <c r="X6" s="58" t="n"/>
+      <c r="Y6" s="58" t="n"/>
+      <c r="Z6" s="58" t="n"/>
+      <c r="AA6" s="58" t="n"/>
+      <c r="AB6" s="58" t="n"/>
+      <c r="AC6" s="58" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="53" t="n"/>
-      <c r="B7" s="53" t="n"/>
-      <c r="C7" s="52" t="n"/>
+      <c r="B7" s="52" t="n"/>
+      <c r="C7" s="53" t="n"/>
       <c r="D7" s="53" t="n"/>
       <c r="E7" s="53" t="n"/>
-      <c r="F7" s="53" t="n"/>
-      <c r="G7" s="53" t="n"/>
-      <c r="H7" s="53" t="n"/>
+      <c r="F7" s="58" t="n"/>
+      <c r="G7" s="58" t="n"/>
+      <c r="H7" s="58" t="n"/>
+      <c r="I7" s="58" t="n"/>
+      <c r="J7" s="58" t="n"/>
+      <c r="K7" s="58" t="n"/>
+      <c r="L7" s="58" t="n"/>
+      <c r="M7" s="58" t="n"/>
+      <c r="N7" s="58" t="n"/>
+      <c r="O7" s="58" t="n"/>
+      <c r="P7" s="58" t="n"/>
+      <c r="Q7" s="58" t="n"/>
+      <c r="R7" s="58" t="n"/>
+      <c r="S7" s="58" t="n"/>
+      <c r="T7" s="53" t="n"/>
+      <c r="U7" s="58" t="n"/>
+      <c r="V7" s="53" t="n"/>
+      <c r="W7" s="53" t="n"/>
+      <c r="X7" s="58" t="n"/>
+      <c r="Y7" s="58" t="n"/>
+      <c r="Z7" s="58" t="n"/>
+      <c r="AA7" s="58" t="n"/>
+      <c r="AB7" s="58" t="n"/>
+      <c r="AC7" s="58" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="53" t="n"/>
-      <c r="B8" s="53" t="n"/>
-      <c r="C8" s="52" t="n"/>
+      <c r="B8" s="52" t="n"/>
+      <c r="C8" s="53" t="n"/>
       <c r="D8" s="53" t="n"/>
       <c r="E8" s="53" t="n"/>
-      <c r="F8" s="53" t="n"/>
-      <c r="G8" s="53" t="n"/>
-      <c r="H8" s="53" t="n"/>
+      <c r="F8" s="58" t="n"/>
+      <c r="G8" s="58" t="n"/>
+      <c r="H8" s="58" t="n"/>
+      <c r="I8" s="58" t="n"/>
+      <c r="J8" s="58" t="n"/>
+      <c r="K8" s="58" t="n"/>
+      <c r="L8" s="58" t="n"/>
+      <c r="M8" s="58" t="n"/>
+      <c r="N8" s="58" t="n"/>
+      <c r="O8" s="58" t="n"/>
+      <c r="P8" s="58" t="n"/>
+      <c r="Q8" s="58" t="n"/>
+      <c r="R8" s="58" t="n"/>
+      <c r="S8" s="58" t="n"/>
+      <c r="T8" s="53" t="n"/>
+      <c r="U8" s="58" t="n"/>
+      <c r="V8" s="53" t="n"/>
+      <c r="W8" s="53" t="n"/>
+      <c r="X8" s="58" t="n"/>
+      <c r="Y8" s="58" t="n"/>
+      <c r="Z8" s="58" t="n"/>
+      <c r="AA8" s="58" t="n"/>
+      <c r="AB8" s="58" t="n"/>
+      <c r="AC8" s="58" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="53" t="n"/>
-      <c r="B9" s="53" t="n"/>
-      <c r="C9" s="52" t="n"/>
+      <c r="B9" s="52" t="n"/>
+      <c r="C9" s="53" t="n"/>
       <c r="D9" s="53" t="n"/>
       <c r="E9" s="53" t="n"/>
-      <c r="F9" s="53" t="n"/>
-      <c r="G9" s="53" t="n"/>
-      <c r="H9" s="53" t="n"/>
+      <c r="F9" s="58" t="n"/>
+      <c r="G9" s="58" t="n"/>
+      <c r="H9" s="58" t="n"/>
+      <c r="I9" s="58" t="n"/>
+      <c r="J9" s="58" t="n"/>
+      <c r="K9" s="58" t="n"/>
+      <c r="L9" s="58" t="n"/>
+      <c r="M9" s="58" t="n"/>
+      <c r="N9" s="58" t="n"/>
+      <c r="O9" s="58" t="n"/>
+      <c r="P9" s="58" t="n"/>
+      <c r="Q9" s="58" t="n"/>
+      <c r="R9" s="58" t="n"/>
+      <c r="S9" s="58" t="n"/>
+      <c r="T9" s="53" t="n"/>
+      <c r="U9" s="58" t="n"/>
+      <c r="V9" s="53" t="n"/>
+      <c r="W9" s="53" t="n"/>
+      <c r="X9" s="58" t="n"/>
+      <c r="Y9" s="58" t="n"/>
+      <c r="Z9" s="58" t="n"/>
+      <c r="AA9" s="58" t="n"/>
+      <c r="AB9" s="58" t="n"/>
+      <c r="AC9" s="58" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="53" t="n"/>
-      <c r="B10" s="53" t="n"/>
-      <c r="C10" s="52" t="n"/>
+      <c r="B10" s="52" t="n"/>
+      <c r="C10" s="53" t="n"/>
       <c r="D10" s="53" t="n"/>
       <c r="E10" s="53" t="n"/>
-      <c r="F10" s="53" t="n"/>
-      <c r="G10" s="53" t="n"/>
-      <c r="H10" s="53" t="n"/>
+      <c r="F10" s="58" t="n"/>
+      <c r="G10" s="58" t="n"/>
+      <c r="H10" s="58" t="n"/>
+      <c r="I10" s="58" t="n"/>
+      <c r="J10" s="58" t="n"/>
+      <c r="K10" s="58" t="n"/>
+      <c r="L10" s="58" t="n"/>
+      <c r="M10" s="58" t="n"/>
+      <c r="N10" s="58" t="n"/>
+      <c r="O10" s="58" t="n"/>
+      <c r="P10" s="58" t="n"/>
+      <c r="Q10" s="58" t="n"/>
+      <c r="R10" s="58" t="n"/>
+      <c r="S10" s="58" t="n"/>
+      <c r="T10" s="53" t="n"/>
+      <c r="U10" s="58" t="n"/>
+      <c r="V10" s="53" t="n"/>
+      <c r="W10" s="53" t="n"/>
+      <c r="X10" s="58" t="n"/>
+      <c r="Y10" s="58" t="n"/>
+      <c r="Z10" s="58" t="n"/>
+      <c r="AA10" s="58" t="n"/>
+      <c r="AB10" s="58" t="n"/>
+      <c r="AC10" s="58" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="53" t="n"/>
-      <c r="B11" s="53" t="n"/>
-      <c r="C11" s="52" t="n"/>
+      <c r="B11" s="52" t="n"/>
+      <c r="C11" s="53" t="n"/>
       <c r="D11" s="53" t="n"/>
       <c r="E11" s="53" t="n"/>
-      <c r="F11" s="53" t="n"/>
-      <c r="G11" s="53" t="n"/>
-      <c r="H11" s="53" t="n"/>
+      <c r="F11" s="58" t="n"/>
+      <c r="G11" s="58" t="n"/>
+      <c r="H11" s="58" t="n"/>
+      <c r="I11" s="58" t="n"/>
+      <c r="J11" s="58" t="n"/>
+      <c r="K11" s="58" t="n"/>
+      <c r="L11" s="58" t="n"/>
+      <c r="M11" s="58" t="n"/>
+      <c r="N11" s="58" t="n"/>
+      <c r="O11" s="58" t="n"/>
+      <c r="P11" s="58" t="n"/>
+      <c r="Q11" s="58" t="n"/>
+      <c r="R11" s="58" t="n"/>
+      <c r="S11" s="58" t="n"/>
+      <c r="T11" s="53" t="n"/>
+      <c r="U11" s="58" t="n"/>
+      <c r="V11" s="53" t="n"/>
+      <c r="W11" s="53" t="n"/>
+      <c r="X11" s="58" t="n"/>
+      <c r="Y11" s="58" t="n"/>
+      <c r="Z11" s="58" t="n"/>
+      <c r="AA11" s="58" t="n"/>
+      <c r="AB11" s="58" t="n"/>
+      <c r="AC11" s="58" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="53" t="n"/>
-      <c r="B12" s="53" t="n"/>
-      <c r="C12" s="52" t="n"/>
+      <c r="B12" s="52" t="n"/>
+      <c r="C12" s="53" t="n"/>
       <c r="D12" s="53" t="n"/>
       <c r="E12" s="53" t="n"/>
-      <c r="F12" s="53" t="n"/>
-      <c r="G12" s="53" t="n"/>
-      <c r="H12" s="53" t="n"/>
+      <c r="F12" s="58" t="n"/>
+      <c r="G12" s="58" t="n"/>
+      <c r="H12" s="58" t="n"/>
+      <c r="I12" s="58" t="n"/>
+      <c r="J12" s="58" t="n"/>
+      <c r="K12" s="58" t="n"/>
+      <c r="L12" s="58" t="n"/>
+      <c r="M12" s="58" t="n"/>
+      <c r="N12" s="58" t="n"/>
+      <c r="O12" s="58" t="n"/>
+      <c r="P12" s="58" t="n"/>
+      <c r="Q12" s="58" t="n"/>
+      <c r="R12" s="58" t="n"/>
+      <c r="S12" s="58" t="n"/>
+      <c r="T12" s="53" t="n"/>
+      <c r="U12" s="58" t="n"/>
+      <c r="V12" s="53" t="n"/>
+      <c r="W12" s="53" t="n"/>
+      <c r="X12" s="58" t="n"/>
+      <c r="Y12" s="58" t="n"/>
+      <c r="Z12" s="58" t="n"/>
+      <c r="AA12" s="58" t="n"/>
+      <c r="AB12" s="58" t="n"/>
+      <c r="AC12" s="58" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="53" t="n"/>
-      <c r="B13" s="53" t="n"/>
-      <c r="C13" s="52" t="n"/>
+      <c r="B13" s="52" t="n"/>
+      <c r="C13" s="53" t="n"/>
       <c r="D13" s="53" t="n"/>
       <c r="E13" s="53" t="n"/>
-      <c r="F13" s="53" t="n"/>
-      <c r="G13" s="53" t="n"/>
-      <c r="H13" s="53" t="n"/>
+      <c r="F13" s="58" t="n"/>
+      <c r="G13" s="58" t="n"/>
+      <c r="H13" s="58" t="n"/>
+      <c r="I13" s="58" t="n"/>
+      <c r="J13" s="58" t="n"/>
+      <c r="K13" s="58" t="n"/>
+      <c r="L13" s="58" t="n"/>
+      <c r="M13" s="58" t="n"/>
+      <c r="N13" s="58" t="n"/>
+      <c r="O13" s="58" t="n"/>
+      <c r="P13" s="58" t="n"/>
+      <c r="Q13" s="58" t="n"/>
+      <c r="R13" s="58" t="n"/>
+      <c r="S13" s="58" t="n"/>
+      <c r="T13" s="53" t="n"/>
+      <c r="U13" s="58" t="n"/>
+      <c r="V13" s="53" t="n"/>
+      <c r="W13" s="53" t="n"/>
+      <c r="X13" s="58" t="n"/>
+      <c r="Y13" s="58" t="n"/>
+      <c r="Z13" s="58" t="n"/>
+      <c r="AA13" s="58" t="n"/>
+      <c r="AB13" s="58" t="n"/>
+      <c r="AC13" s="58" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="53" t="n"/>
-      <c r="B14" s="53" t="n"/>
-      <c r="C14" s="52" t="n"/>
+      <c r="B14" s="52" t="n"/>
+      <c r="C14" s="53" t="n"/>
       <c r="D14" s="53" t="n"/>
       <c r="E14" s="53" t="n"/>
-      <c r="F14" s="53" t="n"/>
-      <c r="G14" s="53" t="n"/>
-      <c r="H14" s="53" t="n"/>
+      <c r="F14" s="58" t="n"/>
+      <c r="G14" s="58" t="n"/>
+      <c r="H14" s="58" t="n"/>
+      <c r="I14" s="58" t="n"/>
+      <c r="J14" s="58" t="n"/>
+      <c r="K14" s="58" t="n"/>
+      <c r="L14" s="58" t="n"/>
+      <c r="M14" s="58" t="n"/>
+      <c r="N14" s="58" t="n"/>
+      <c r="O14" s="58" t="n"/>
+      <c r="P14" s="58" t="n"/>
+      <c r="Q14" s="58" t="n"/>
+      <c r="R14" s="58" t="n"/>
+      <c r="S14" s="58" t="n"/>
+      <c r="T14" s="53" t="n"/>
+      <c r="U14" s="58" t="n"/>
+      <c r="V14" s="53" t="n"/>
+      <c r="W14" s="53" t="n"/>
+      <c r="X14" s="58" t="n"/>
+      <c r="Y14" s="58" t="n"/>
+      <c r="Z14" s="58" t="n"/>
+      <c r="AA14" s="58" t="n"/>
+      <c r="AB14" s="58" t="n"/>
+      <c r="AC14" s="58" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="53" t="n"/>
-      <c r="B15" s="53" t="n"/>
-      <c r="C15" s="52" t="n"/>
+      <c r="B15" s="52" t="n"/>
+      <c r="C15" s="53" t="n"/>
       <c r="D15" s="53" t="n"/>
       <c r="E15" s="53" t="n"/>
-      <c r="F15" s="53" t="n"/>
-      <c r="G15" s="53" t="n"/>
-      <c r="H15" s="53" t="n"/>
+      <c r="F15" s="58" t="n"/>
+      <c r="G15" s="58" t="n"/>
+      <c r="H15" s="58" t="n"/>
+      <c r="I15" s="58" t="n"/>
+      <c r="J15" s="58" t="n"/>
+      <c r="K15" s="58" t="n"/>
+      <c r="L15" s="58" t="n"/>
+      <c r="M15" s="58" t="n"/>
+      <c r="N15" s="58" t="n"/>
+      <c r="O15" s="58" t="n"/>
+      <c r="P15" s="58" t="n"/>
+      <c r="Q15" s="58" t="n"/>
+      <c r="R15" s="58" t="n"/>
+      <c r="S15" s="58" t="n"/>
+      <c r="T15" s="53" t="n"/>
+      <c r="U15" s="58" t="n"/>
+      <c r="V15" s="53" t="n"/>
+      <c r="W15" s="53" t="n"/>
+      <c r="X15" s="58" t="n"/>
+      <c r="Y15" s="58" t="n"/>
+      <c r="Z15" s="58" t="n"/>
+      <c r="AA15" s="58" t="n"/>
+      <c r="AB15" s="58" t="n"/>
+      <c r="AC15" s="58" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="53" t="n"/>
-      <c r="B16" s="53" t="n"/>
-      <c r="C16" s="52" t="n"/>
+      <c r="B16" s="52" t="n"/>
+      <c r="C16" s="53" t="n"/>
       <c r="D16" s="53" t="n"/>
       <c r="E16" s="53" t="n"/>
-      <c r="F16" s="53" t="n"/>
-      <c r="G16" s="53" t="n"/>
-      <c r="H16" s="53" t="n"/>
+      <c r="F16" s="58" t="n"/>
+      <c r="G16" s="58" t="n"/>
+      <c r="H16" s="58" t="n"/>
+      <c r="I16" s="58" t="n"/>
+      <c r="J16" s="58" t="n"/>
+      <c r="K16" s="58" t="n"/>
+      <c r="L16" s="58" t="n"/>
+      <c r="M16" s="58" t="n"/>
+      <c r="N16" s="58" t="n"/>
+      <c r="O16" s="58" t="n"/>
+      <c r="P16" s="58" t="n"/>
+      <c r="Q16" s="58" t="n"/>
+      <c r="R16" s="58" t="n"/>
+      <c r="S16" s="58" t="n"/>
+      <c r="T16" s="53" t="n"/>
+      <c r="U16" s="58" t="n"/>
+      <c r="V16" s="53" t="n"/>
+      <c r="W16" s="53" t="n"/>
+      <c r="X16" s="58" t="n"/>
+      <c r="Y16" s="58" t="n"/>
+      <c r="Z16" s="58" t="n"/>
+      <c r="AA16" s="58" t="n"/>
+      <c r="AB16" s="58" t="n"/>
+      <c r="AC16" s="58" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="53" t="n"/>
-      <c r="B17" s="53" t="n"/>
-      <c r="C17" s="52" t="n"/>
+      <c r="B17" s="52" t="n"/>
+      <c r="C17" s="53" t="n"/>
       <c r="D17" s="53" t="n"/>
       <c r="E17" s="53" t="n"/>
-      <c r="F17" s="53" t="n"/>
-      <c r="G17" s="53" t="n"/>
-      <c r="H17" s="53" t="n"/>
+      <c r="F17" s="58" t="n"/>
+      <c r="G17" s="58" t="n"/>
+      <c r="H17" s="58" t="n"/>
+      <c r="I17" s="58" t="n"/>
+      <c r="J17" s="58" t="n"/>
+      <c r="K17" s="58" t="n"/>
+      <c r="L17" s="58" t="n"/>
+      <c r="M17" s="58" t="n"/>
+      <c r="N17" s="58" t="n"/>
+      <c r="O17" s="58" t="n"/>
+      <c r="P17" s="58" t="n"/>
+      <c r="Q17" s="58" t="n"/>
+      <c r="R17" s="58" t="n"/>
+      <c r="S17" s="58" t="n"/>
+      <c r="T17" s="53" t="n"/>
+      <c r="U17" s="58" t="n"/>
+      <c r="V17" s="53" t="n"/>
+      <c r="W17" s="53" t="n"/>
+      <c r="X17" s="58" t="n"/>
+      <c r="Y17" s="58" t="n"/>
+      <c r="Z17" s="58" t="n"/>
+      <c r="AA17" s="58" t="n"/>
+      <c r="AB17" s="58" t="n"/>
+      <c r="AC17" s="58" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="53" t="n"/>
-      <c r="B18" s="53" t="n"/>
-      <c r="C18" s="52" t="n"/>
+      <c r="B18" s="52" t="n"/>
+      <c r="C18" s="53" t="n"/>
       <c r="D18" s="53" t="n"/>
       <c r="E18" s="53" t="n"/>
-      <c r="F18" s="53" t="n"/>
-      <c r="G18" s="53" t="n"/>
-      <c r="H18" s="53" t="n"/>
+      <c r="F18" s="58" t="n"/>
+      <c r="G18" s="58" t="n"/>
+      <c r="H18" s="58" t="n"/>
+      <c r="I18" s="58" t="n"/>
+      <c r="J18" s="58" t="n"/>
+      <c r="K18" s="58" t="n"/>
+      <c r="L18" s="58" t="n"/>
+      <c r="M18" s="58" t="n"/>
+      <c r="N18" s="58" t="n"/>
+      <c r="O18" s="58" t="n"/>
+      <c r="P18" s="58" t="n"/>
+      <c r="Q18" s="58" t="n"/>
+      <c r="R18" s="58" t="n"/>
+      <c r="S18" s="58" t="n"/>
+      <c r="T18" s="53" t="n"/>
+      <c r="U18" s="58" t="n"/>
+      <c r="V18" s="53" t="n"/>
+      <c r="W18" s="53" t="n"/>
+      <c r="X18" s="58" t="n"/>
+      <c r="Y18" s="58" t="n"/>
+      <c r="Z18" s="58" t="n"/>
+      <c r="AA18" s="58" t="n"/>
+      <c r="AB18" s="58" t="n"/>
+      <c r="AC18" s="58" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="53" t="n"/>
-      <c r="B19" s="53" t="n"/>
-      <c r="C19" s="52" t="n"/>
+      <c r="B19" s="52" t="n"/>
+      <c r="C19" s="53" t="n"/>
       <c r="D19" s="53" t="n"/>
       <c r="E19" s="53" t="n"/>
-      <c r="F19" s="53" t="n"/>
-      <c r="G19" s="53" t="n"/>
-      <c r="H19" s="53" t="n"/>
+      <c r="F19" s="58" t="n"/>
+      <c r="G19" s="58" t="n"/>
+      <c r="H19" s="58" t="n"/>
+      <c r="I19" s="58" t="n"/>
+      <c r="J19" s="58" t="n"/>
+      <c r="K19" s="58" t="n"/>
+      <c r="L19" s="58" t="n"/>
+      <c r="M19" s="58" t="n"/>
+      <c r="N19" s="58" t="n"/>
+      <c r="O19" s="58" t="n"/>
+      <c r="P19" s="58" t="n"/>
+      <c r="Q19" s="58" t="n"/>
+      <c r="R19" s="58" t="n"/>
+      <c r="S19" s="58" t="n"/>
+      <c r="T19" s="53" t="n"/>
+      <c r="U19" s="58" t="n"/>
+      <c r="V19" s="53" t="n"/>
+      <c r="W19" s="53" t="n"/>
+      <c r="X19" s="58" t="n"/>
+      <c r="Y19" s="58" t="n"/>
+      <c r="Z19" s="58" t="n"/>
+      <c r="AA19" s="58" t="n"/>
+      <c r="AB19" s="58" t="n"/>
+      <c r="AC19" s="58" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="53" t="n"/>
-      <c r="B20" s="53" t="n"/>
-      <c r="C20" s="52" t="n"/>
+      <c r="B20" s="52" t="n"/>
+      <c r="C20" s="53" t="n"/>
       <c r="D20" s="53" t="n"/>
       <c r="E20" s="53" t="n"/>
-      <c r="F20" s="53" t="n"/>
-      <c r="G20" s="53" t="n"/>
-      <c r="H20" s="53" t="n"/>
+      <c r="F20" s="58" t="n"/>
+      <c r="G20" s="58" t="n"/>
+      <c r="H20" s="58" t="n"/>
+      <c r="I20" s="58" t="n"/>
+      <c r="J20" s="58" t="n"/>
+      <c r="K20" s="58" t="n"/>
+      <c r="L20" s="58" t="n"/>
+      <c r="M20" s="58" t="n"/>
+      <c r="N20" s="58" t="n"/>
+      <c r="O20" s="58" t="n"/>
+      <c r="P20" s="58" t="n"/>
+      <c r="Q20" s="58" t="n"/>
+      <c r="R20" s="58" t="n"/>
+      <c r="S20" s="58" t="n"/>
+      <c r="T20" s="53" t="n"/>
+      <c r="U20" s="58" t="n"/>
+      <c r="V20" s="53" t="n"/>
+      <c r="W20" s="53" t="n"/>
+      <c r="X20" s="58" t="n"/>
+      <c r="Y20" s="58" t="n"/>
+      <c r="Z20" s="58" t="n"/>
+      <c r="AA20" s="58" t="n"/>
+      <c r="AB20" s="58" t="n"/>
+      <c r="AC20" s="58" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="53" t="n"/>
-      <c r="B21" s="53" t="n"/>
-      <c r="C21" s="52" t="n"/>
+      <c r="B21" s="52" t="n"/>
+      <c r="C21" s="53" t="n"/>
       <c r="D21" s="53" t="n"/>
       <c r="E21" s="53" t="n"/>
-      <c r="F21" s="53" t="n"/>
-      <c r="G21" s="53" t="n"/>
-      <c r="H21" s="53" t="n"/>
+      <c r="F21" s="58" t="n"/>
+      <c r="G21" s="58" t="n"/>
+      <c r="H21" s="58" t="n"/>
+      <c r="I21" s="58" t="n"/>
+      <c r="J21" s="58" t="n"/>
+      <c r="K21" s="58" t="n"/>
+      <c r="L21" s="58" t="n"/>
+      <c r="M21" s="58" t="n"/>
+      <c r="N21" s="58" t="n"/>
+      <c r="O21" s="58" t="n"/>
+      <c r="P21" s="58" t="n"/>
+      <c r="Q21" s="58" t="n"/>
+      <c r="R21" s="58" t="n"/>
+      <c r="S21" s="58" t="n"/>
+      <c r="T21" s="53" t="n"/>
+      <c r="U21" s="58" t="n"/>
+      <c r="V21" s="53" t="n"/>
+      <c r="W21" s="53" t="n"/>
+      <c r="X21" s="58" t="n"/>
+      <c r="Y21" s="58" t="n"/>
+      <c r="Z21" s="58" t="n"/>
+      <c r="AA21" s="58" t="n"/>
+      <c r="AB21" s="58" t="n"/>
+      <c r="AC21" s="58" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="53" t="n"/>
-      <c r="B22" s="53" t="n"/>
-      <c r="C22" s="52" t="n"/>
+      <c r="B22" s="52" t="n"/>
+      <c r="C22" s="53" t="n"/>
       <c r="D22" s="53" t="n"/>
       <c r="E22" s="53" t="n"/>
-      <c r="F22" s="53" t="n"/>
-      <c r="G22" s="53" t="n"/>
-      <c r="H22" s="53" t="n"/>
+      <c r="F22" s="58" t="n"/>
+      <c r="G22" s="58" t="n"/>
+      <c r="H22" s="58" t="n"/>
+      <c r="I22" s="58" t="n"/>
+      <c r="J22" s="58" t="n"/>
+      <c r="K22" s="58" t="n"/>
+      <c r="L22" s="58" t="n"/>
+      <c r="M22" s="58" t="n"/>
+      <c r="N22" s="58" t="n"/>
+      <c r="O22" s="58" t="n"/>
+      <c r="P22" s="58" t="n"/>
+      <c r="Q22" s="58" t="n"/>
+      <c r="R22" s="58" t="n"/>
+      <c r="S22" s="58" t="n"/>
+      <c r="T22" s="53" t="n"/>
+      <c r="U22" s="58" t="n"/>
+      <c r="V22" s="53" t="n"/>
+      <c r="W22" s="53" t="n"/>
+      <c r="X22" s="58" t="n"/>
+      <c r="Y22" s="58" t="n"/>
+      <c r="Z22" s="58" t="n"/>
+      <c r="AA22" s="58" t="n"/>
+      <c r="AB22" s="58" t="n"/>
+      <c r="AC22" s="58" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="53" t="n"/>
-      <c r="B23" s="53" t="n"/>
-      <c r="C23" s="52" t="n"/>
+      <c r="B23" s="52" t="n"/>
+      <c r="C23" s="53" t="n"/>
       <c r="D23" s="53" t="n"/>
       <c r="E23" s="53" t="n"/>
-      <c r="F23" s="53" t="n"/>
-      <c r="G23" s="53" t="n"/>
-      <c r="H23" s="53" t="n"/>
+      <c r="F23" s="58" t="n"/>
+      <c r="G23" s="58" t="n"/>
+      <c r="H23" s="58" t="n"/>
+      <c r="I23" s="58" t="n"/>
+      <c r="J23" s="58" t="n"/>
+      <c r="K23" s="58" t="n"/>
+      <c r="L23" s="58" t="n"/>
+      <c r="M23" s="58" t="n"/>
+      <c r="N23" s="58" t="n"/>
+      <c r="O23" s="58" t="n"/>
+      <c r="P23" s="58" t="n"/>
+      <c r="Q23" s="58" t="n"/>
+      <c r="R23" s="58" t="n"/>
+      <c r="S23" s="58" t="n"/>
+      <c r="T23" s="53" t="n"/>
+      <c r="U23" s="58" t="n"/>
+      <c r="V23" s="53" t="n"/>
+      <c r="W23" s="53" t="n"/>
+      <c r="X23" s="58" t="n"/>
+      <c r="Y23" s="58" t="n"/>
+      <c r="Z23" s="58" t="n"/>
+      <c r="AA23" s="58" t="n"/>
+      <c r="AB23" s="58" t="n"/>
+      <c r="AC23" s="58" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="53" t="n"/>
-      <c r="B24" s="53" t="n"/>
-      <c r="C24" s="52" t="n"/>
+      <c r="B24" s="52" t="n"/>
+      <c r="C24" s="53" t="n"/>
       <c r="D24" s="53" t="n"/>
       <c r="E24" s="53" t="n"/>
-      <c r="F24" s="53" t="n"/>
-      <c r="G24" s="53" t="n"/>
-      <c r="H24" s="53" t="n"/>
+      <c r="F24" s="58" t="n"/>
+      <c r="G24" s="58" t="n"/>
+      <c r="H24" s="58" t="n"/>
+      <c r="I24" s="58" t="n"/>
+      <c r="J24" s="58" t="n"/>
+      <c r="K24" s="58" t="n"/>
+      <c r="L24" s="58" t="n"/>
+      <c r="M24" s="58" t="n"/>
+      <c r="N24" s="58" t="n"/>
+      <c r="O24" s="58" t="n"/>
+      <c r="P24" s="58" t="n"/>
+      <c r="Q24" s="58" t="n"/>
+      <c r="R24" s="58" t="n"/>
+      <c r="S24" s="58" t="n"/>
+      <c r="T24" s="53" t="n"/>
+      <c r="U24" s="58" t="n"/>
+      <c r="V24" s="53" t="n"/>
+      <c r="W24" s="53" t="n"/>
+      <c r="X24" s="58" t="n"/>
+      <c r="Y24" s="58" t="n"/>
+      <c r="Z24" s="58" t="n"/>
+      <c r="AA24" s="58" t="n"/>
+      <c r="AB24" s="58" t="n"/>
+      <c r="AC24" s="58" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="53" t="n"/>
-      <c r="B25" s="53" t="n"/>
-      <c r="C25" s="52" t="n"/>
+      <c r="B25" s="52" t="n"/>
+      <c r="C25" s="53" t="n"/>
       <c r="D25" s="53" t="n"/>
       <c r="E25" s="53" t="n"/>
-      <c r="F25" s="53" t="n"/>
-      <c r="G25" s="53" t="n"/>
-      <c r="H25" s="53" t="n"/>
+      <c r="F25" s="58" t="n"/>
+      <c r="G25" s="58" t="n"/>
+      <c r="H25" s="58" t="n"/>
+      <c r="I25" s="58" t="n"/>
+      <c r="J25" s="58" t="n"/>
+      <c r="K25" s="58" t="n"/>
+      <c r="L25" s="58" t="n"/>
+      <c r="M25" s="58" t="n"/>
+      <c r="N25" s="58" t="n"/>
+      <c r="O25" s="58" t="n"/>
+      <c r="P25" s="58" t="n"/>
+      <c r="Q25" s="58" t="n"/>
+      <c r="R25" s="58" t="n"/>
+      <c r="S25" s="58" t="n"/>
+      <c r="T25" s="53" t="n"/>
+      <c r="U25" s="58" t="n"/>
+      <c r="V25" s="53" t="n"/>
+      <c r="W25" s="53" t="n"/>
+      <c r="X25" s="58" t="n"/>
+      <c r="Y25" s="58" t="n"/>
+      <c r="Z25" s="58" t="n"/>
+      <c r="AA25" s="58" t="n"/>
+      <c r="AB25" s="58" t="n"/>
+      <c r="AC25" s="58" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="53" t="n"/>
-      <c r="B26" s="53" t="n"/>
-      <c r="C26" s="52" t="n"/>
+      <c r="B26" s="52" t="n"/>
+      <c r="C26" s="53" t="n"/>
       <c r="D26" s="53" t="n"/>
       <c r="E26" s="53" t="n"/>
-      <c r="F26" s="53" t="n"/>
-      <c r="G26" s="53" t="n"/>
-      <c r="H26" s="53" t="n"/>
+      <c r="F26" s="58" t="n"/>
+      <c r="G26" s="58" t="n"/>
+      <c r="H26" s="58" t="n"/>
+      <c r="I26" s="58" t="n"/>
+      <c r="J26" s="58" t="n"/>
+      <c r="K26" s="58" t="n"/>
+      <c r="L26" s="58" t="n"/>
+      <c r="M26" s="58" t="n"/>
+      <c r="N26" s="58" t="n"/>
+      <c r="O26" s="58" t="n"/>
+      <c r="P26" s="58" t="n"/>
+      <c r="Q26" s="58" t="n"/>
+      <c r="R26" s="58" t="n"/>
+      <c r="S26" s="58" t="n"/>
+      <c r="T26" s="53" t="n"/>
+      <c r="U26" s="58" t="n"/>
+      <c r="V26" s="53" t="n"/>
+      <c r="W26" s="53" t="n"/>
+      <c r="X26" s="58" t="n"/>
+      <c r="Y26" s="58" t="n"/>
+      <c r="Z26" s="58" t="n"/>
+      <c r="AA26" s="58" t="n"/>
+      <c r="AB26" s="58" t="n"/>
+      <c r="AC26" s="58" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="53" t="n"/>
-      <c r="B27" s="53" t="n"/>
-      <c r="C27" s="52" t="n"/>
+      <c r="B27" s="52" t="n"/>
+      <c r="C27" s="53" t="n"/>
       <c r="D27" s="53" t="n"/>
       <c r="E27" s="53" t="n"/>
-      <c r="F27" s="53" t="n"/>
-      <c r="G27" s="53" t="n"/>
-      <c r="H27" s="53" t="n"/>
+      <c r="F27" s="58" t="n"/>
+      <c r="G27" s="58" t="n"/>
+      <c r="H27" s="58" t="n"/>
+      <c r="I27" s="58" t="n"/>
+      <c r="J27" s="58" t="n"/>
+      <c r="K27" s="58" t="n"/>
+      <c r="L27" s="58" t="n"/>
+      <c r="M27" s="58" t="n"/>
+      <c r="N27" s="58" t="n"/>
+      <c r="O27" s="58" t="n"/>
+      <c r="P27" s="58" t="n"/>
+      <c r="Q27" s="58" t="n"/>
+      <c r="R27" s="58" t="n"/>
+      <c r="S27" s="58" t="n"/>
+      <c r="T27" s="53" t="n"/>
+      <c r="U27" s="58" t="n"/>
+      <c r="V27" s="53" t="n"/>
+      <c r="W27" s="53" t="n"/>
+      <c r="X27" s="58" t="n"/>
+      <c r="Y27" s="58" t="n"/>
+      <c r="Z27" s="58" t="n"/>
+      <c r="AA27" s="58" t="n"/>
+      <c r="AB27" s="58" t="n"/>
+      <c r="AC27" s="58" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="53" t="n"/>
-      <c r="B28" s="53" t="n"/>
-      <c r="C28" s="52" t="n"/>
+      <c r="B28" s="52" t="n"/>
+      <c r="C28" s="53" t="n"/>
       <c r="D28" s="53" t="n"/>
       <c r="E28" s="53" t="n"/>
-      <c r="F28" s="53" t="n"/>
-      <c r="G28" s="53" t="n"/>
-      <c r="H28" s="53" t="n"/>
+      <c r="F28" s="58" t="n"/>
+      <c r="G28" s="58" t="n"/>
+      <c r="H28" s="58" t="n"/>
+      <c r="I28" s="58" t="n"/>
+      <c r="J28" s="58" t="n"/>
+      <c r="K28" s="58" t="n"/>
+      <c r="L28" s="58" t="n"/>
+      <c r="M28" s="58" t="n"/>
+      <c r="N28" s="58" t="n"/>
+      <c r="O28" s="58" t="n"/>
+      <c r="P28" s="58" t="n"/>
+      <c r="Q28" s="58" t="n"/>
+      <c r="R28" s="58" t="n"/>
+      <c r="S28" s="58" t="n"/>
+      <c r="T28" s="53" t="n"/>
+      <c r="U28" s="58" t="n"/>
+      <c r="V28" s="53" t="n"/>
+      <c r="W28" s="53" t="n"/>
+      <c r="X28" s="58" t="n"/>
+      <c r="Y28" s="58" t="n"/>
+      <c r="Z28" s="58" t="n"/>
+      <c r="AA28" s="58" t="n"/>
+      <c r="AB28" s="58" t="n"/>
+      <c r="AC28" s="58" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="53" t="n"/>
-      <c r="B29" s="53" t="n"/>
-      <c r="C29" s="52" t="n"/>
+      <c r="B29" s="52" t="n"/>
+      <c r="C29" s="53" t="n"/>
       <c r="D29" s="53" t="n"/>
       <c r="E29" s="53" t="n"/>
-      <c r="F29" s="53" t="n"/>
-      <c r="G29" s="53" t="n"/>
-      <c r="H29" s="53" t="n"/>
+      <c r="F29" s="58" t="n"/>
+      <c r="G29" s="58" t="n"/>
+      <c r="H29" s="58" t="n"/>
+      <c r="I29" s="58" t="n"/>
+      <c r="J29" s="58" t="n"/>
+      <c r="K29" s="58" t="n"/>
+      <c r="L29" s="58" t="n"/>
+      <c r="M29" s="58" t="n"/>
+      <c r="N29" s="58" t="n"/>
+      <c r="O29" s="58" t="n"/>
+      <c r="P29" s="58" t="n"/>
+      <c r="Q29" s="58" t="n"/>
+      <c r="R29" s="58" t="n"/>
+      <c r="S29" s="58" t="n"/>
+      <c r="T29" s="53" t="n"/>
+      <c r="U29" s="58" t="n"/>
+      <c r="V29" s="53" t="n"/>
+      <c r="W29" s="53" t="n"/>
+      <c r="X29" s="58" t="n"/>
+      <c r="Y29" s="58" t="n"/>
+      <c r="Z29" s="58" t="n"/>
+      <c r="AA29" s="58" t="n"/>
+      <c r="AB29" s="58" t="n"/>
+      <c r="AC29" s="58" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="53" t="n"/>
-      <c r="B30" s="53" t="n"/>
-      <c r="C30" s="52" t="n"/>
+      <c r="B30" s="52" t="n"/>
+      <c r="C30" s="53" t="n"/>
       <c r="D30" s="53" t="n"/>
       <c r="E30" s="53" t="n"/>
-      <c r="F30" s="53" t="n"/>
-      <c r="G30" s="53" t="n"/>
-      <c r="H30" s="53" t="n"/>
+      <c r="F30" s="58" t="n"/>
+      <c r="G30" s="58" t="n"/>
+      <c r="H30" s="58" t="n"/>
+      <c r="I30" s="58" t="n"/>
+      <c r="J30" s="58" t="n"/>
+      <c r="K30" s="58" t="n"/>
+      <c r="L30" s="58" t="n"/>
+      <c r="M30" s="58" t="n"/>
+      <c r="N30" s="58" t="n"/>
+      <c r="O30" s="58" t="n"/>
+      <c r="P30" s="58" t="n"/>
+      <c r="Q30" s="58" t="n"/>
+      <c r="R30" s="58" t="n"/>
+      <c r="S30" s="58" t="n"/>
+      <c r="T30" s="53" t="n"/>
+      <c r="U30" s="58" t="n"/>
+      <c r="V30" s="53" t="n"/>
+      <c r="W30" s="53" t="n"/>
+      <c r="X30" s="58" t="n"/>
+      <c r="Y30" s="58" t="n"/>
+      <c r="Z30" s="58" t="n"/>
+      <c r="AA30" s="58" t="n"/>
+      <c r="AB30" s="58" t="n"/>
+      <c r="AC30" s="58" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="53" t="n"/>
-      <c r="B31" s="53" t="n"/>
-      <c r="C31" s="52" t="n"/>
+      <c r="B31" s="52" t="n"/>
+      <c r="C31" s="53" t="n"/>
       <c r="D31" s="53" t="n"/>
       <c r="E31" s="53" t="n"/>
-      <c r="F31" s="53" t="n"/>
-      <c r="G31" s="53" t="n"/>
-      <c r="H31" s="53" t="n"/>
+      <c r="F31" s="58" t="n"/>
+      <c r="G31" s="58" t="n"/>
+      <c r="H31" s="58" t="n"/>
+      <c r="I31" s="58" t="n"/>
+      <c r="J31" s="58" t="n"/>
+      <c r="K31" s="58" t="n"/>
+      <c r="L31" s="58" t="n"/>
+      <c r="M31" s="58" t="n"/>
+      <c r="N31" s="58" t="n"/>
+      <c r="O31" s="58" t="n"/>
+      <c r="P31" s="58" t="n"/>
+      <c r="Q31" s="58" t="n"/>
+      <c r="R31" s="58" t="n"/>
+      <c r="S31" s="58" t="n"/>
+      <c r="T31" s="53" t="n"/>
+      <c r="U31" s="58" t="n"/>
+      <c r="V31" s="53" t="n"/>
+      <c r="W31" s="53" t="n"/>
+      <c r="X31" s="58" t="n"/>
+      <c r="Y31" s="58" t="n"/>
+      <c r="Z31" s="58" t="n"/>
+      <c r="AA31" s="58" t="n"/>
+      <c r="AB31" s="58" t="n"/>
+      <c r="AC31" s="58" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="53" t="n"/>
-      <c r="B32" s="53" t="n"/>
-      <c r="C32" s="52" t="n"/>
+      <c r="B32" s="52" t="n"/>
+      <c r="C32" s="53" t="n"/>
       <c r="D32" s="53" t="n"/>
       <c r="E32" s="53" t="n"/>
-      <c r="F32" s="53" t="n"/>
-      <c r="G32" s="53" t="n"/>
-      <c r="H32" s="53" t="n"/>
+      <c r="F32" s="58" t="n"/>
+      <c r="G32" s="58" t="n"/>
+      <c r="H32" s="58" t="n"/>
+      <c r="I32" s="58" t="n"/>
+      <c r="J32" s="58" t="n"/>
+      <c r="K32" s="58" t="n"/>
+      <c r="L32" s="58" t="n"/>
+      <c r="M32" s="58" t="n"/>
+      <c r="N32" s="58" t="n"/>
+      <c r="O32" s="58" t="n"/>
+      <c r="P32" s="58" t="n"/>
+      <c r="Q32" s="58" t="n"/>
+      <c r="R32" s="58" t="n"/>
+      <c r="S32" s="58" t="n"/>
+      <c r="T32" s="53" t="n"/>
+      <c r="U32" s="58" t="n"/>
+      <c r="V32" s="53" t="n"/>
+      <c r="W32" s="53" t="n"/>
+      <c r="X32" s="58" t="n"/>
+      <c r="Y32" s="58" t="n"/>
+      <c r="Z32" s="58" t="n"/>
+      <c r="AA32" s="58" t="n"/>
+      <c r="AB32" s="58" t="n"/>
+      <c r="AC32" s="58" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="53" t="n"/>
-      <c r="B33" s="53" t="n"/>
-      <c r="C33" s="52" t="n"/>
+      <c r="B33" s="52" t="n"/>
+      <c r="C33" s="53" t="n"/>
       <c r="D33" s="53" t="n"/>
       <c r="E33" s="53" t="n"/>
-      <c r="F33" s="53" t="n"/>
-      <c r="G33" s="53" t="n"/>
-      <c r="H33" s="53" t="n"/>
+      <c r="F33" s="58" t="n"/>
+      <c r="G33" s="58" t="n"/>
+      <c r="H33" s="58" t="n"/>
+      <c r="I33" s="58" t="n"/>
+      <c r="J33" s="58" t="n"/>
+      <c r="K33" s="58" t="n"/>
+      <c r="L33" s="58" t="n"/>
+      <c r="M33" s="58" t="n"/>
+      <c r="N33" s="58" t="n"/>
+      <c r="O33" s="58" t="n"/>
+      <c r="P33" s="58" t="n"/>
+      <c r="Q33" s="58" t="n"/>
+      <c r="R33" s="58" t="n"/>
+      <c r="S33" s="58" t="n"/>
+      <c r="T33" s="53" t="n"/>
+      <c r="U33" s="58" t="n"/>
+      <c r="V33" s="53" t="n"/>
+      <c r="W33" s="53" t="n"/>
+      <c r="X33" s="58" t="n"/>
+      <c r="Y33" s="58" t="n"/>
+      <c r="Z33" s="58" t="n"/>
+      <c r="AA33" s="58" t="n"/>
+      <c r="AB33" s="58" t="n"/>
+      <c r="AC33" s="58" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="53" t="n"/>
-      <c r="B34" s="53" t="n"/>
-      <c r="C34" s="52" t="n"/>
+      <c r="B34" s="52" t="n"/>
+      <c r="C34" s="53" t="n"/>
       <c r="D34" s="53" t="n"/>
       <c r="E34" s="53" t="n"/>
-      <c r="F34" s="53" t="n"/>
-      <c r="G34" s="53" t="n"/>
-      <c r="H34" s="53" t="n"/>
+      <c r="F34" s="58" t="n"/>
+      <c r="G34" s="58" t="n"/>
+      <c r="H34" s="58" t="n"/>
+      <c r="I34" s="58" t="n"/>
+      <c r="J34" s="58" t="n"/>
+      <c r="K34" s="58" t="n"/>
+      <c r="L34" s="58" t="n"/>
+      <c r="M34" s="58" t="n"/>
+      <c r="N34" s="58" t="n"/>
+      <c r="O34" s="58" t="n"/>
+      <c r="P34" s="58" t="n"/>
+      <c r="Q34" s="58" t="n"/>
+      <c r="R34" s="58" t="n"/>
+      <c r="S34" s="58" t="n"/>
+      <c r="T34" s="53" t="n"/>
+      <c r="U34" s="58" t="n"/>
+      <c r="V34" s="53" t="n"/>
+      <c r="W34" s="53" t="n"/>
+      <c r="X34" s="58" t="n"/>
+      <c r="Y34" s="58" t="n"/>
+      <c r="Z34" s="58" t="n"/>
+      <c r="AA34" s="58" t="n"/>
+      <c r="AB34" s="58" t="n"/>
+      <c r="AC34" s="58" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="53" t="n"/>
-      <c r="B35" s="53" t="n"/>
-      <c r="C35" s="52" t="n"/>
+      <c r="B35" s="52" t="n"/>
+      <c r="C35" s="53" t="n"/>
       <c r="D35" s="53" t="n"/>
       <c r="E35" s="53" t="n"/>
-      <c r="F35" s="53" t="n"/>
-      <c r="G35" s="53" t="n"/>
-      <c r="H35" s="53" t="n"/>
+      <c r="F35" s="58" t="n"/>
+      <c r="G35" s="58" t="n"/>
+      <c r="H35" s="58" t="n"/>
+      <c r="I35" s="58" t="n"/>
+      <c r="J35" s="58" t="n"/>
+      <c r="K35" s="58" t="n"/>
+      <c r="L35" s="58" t="n"/>
+      <c r="M35" s="58" t="n"/>
+      <c r="N35" s="58" t="n"/>
+      <c r="O35" s="58" t="n"/>
+      <c r="P35" s="58" t="n"/>
+      <c r="Q35" s="58" t="n"/>
+      <c r="R35" s="58" t="n"/>
+      <c r="S35" s="58" t="n"/>
+      <c r="T35" s="53" t="n"/>
+      <c r="U35" s="58" t="n"/>
+      <c r="V35" s="53" t="n"/>
+      <c r="W35" s="53" t="n"/>
+      <c r="X35" s="58" t="n"/>
+      <c r="Y35" s="58" t="n"/>
+      <c r="Z35" s="58" t="n"/>
+      <c r="AA35" s="58" t="n"/>
+      <c r="AB35" s="58" t="n"/>
+      <c r="AC35" s="58" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="53" t="n"/>
-      <c r="B36" s="53" t="n"/>
-      <c r="C36" s="52" t="n"/>
+      <c r="B36" s="52" t="n"/>
+      <c r="C36" s="53" t="n"/>
       <c r="D36" s="53" t="n"/>
       <c r="E36" s="53" t="n"/>
-      <c r="F36" s="53" t="n"/>
-      <c r="G36" s="53" t="n"/>
-      <c r="H36" s="53" t="n"/>
+      <c r="F36" s="58" t="n"/>
+      <c r="G36" s="58" t="n"/>
+      <c r="H36" s="58" t="n"/>
+      <c r="I36" s="58" t="n"/>
+      <c r="J36" s="58" t="n"/>
+      <c r="K36" s="58" t="n"/>
+      <c r="L36" s="58" t="n"/>
+      <c r="M36" s="58" t="n"/>
+      <c r="N36" s="58" t="n"/>
+      <c r="O36" s="58" t="n"/>
+      <c r="P36" s="58" t="n"/>
+      <c r="Q36" s="58" t="n"/>
+      <c r="R36" s="58" t="n"/>
+      <c r="S36" s="58" t="n"/>
+      <c r="T36" s="53" t="n"/>
+      <c r="U36" s="58" t="n"/>
+      <c r="V36" s="53" t="n"/>
+      <c r="W36" s="53" t="n"/>
+      <c r="X36" s="58" t="n"/>
+      <c r="Y36" s="58" t="n"/>
+      <c r="Z36" s="58" t="n"/>
+      <c r="AA36" s="58" t="n"/>
+      <c r="AB36" s="58" t="n"/>
+      <c r="AC36" s="58" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="53" t="n"/>
-      <c r="B37" s="53" t="n"/>
-      <c r="C37" s="52" t="n"/>
+      <c r="B37" s="52" t="n"/>
+      <c r="C37" s="53" t="n"/>
       <c r="D37" s="53" t="n"/>
       <c r="E37" s="53" t="n"/>
-      <c r="F37" s="53" t="n"/>
-      <c r="G37" s="53" t="n"/>
-      <c r="H37" s="53" t="n"/>
+      <c r="F37" s="58" t="n"/>
+      <c r="G37" s="58" t="n"/>
+      <c r="H37" s="58" t="n"/>
+      <c r="I37" s="58" t="n"/>
+      <c r="J37" s="58" t="n"/>
+      <c r="K37" s="58" t="n"/>
+      <c r="L37" s="58" t="n"/>
+      <c r="M37" s="58" t="n"/>
+      <c r="N37" s="58" t="n"/>
+      <c r="O37" s="58" t="n"/>
+      <c r="P37" s="58" t="n"/>
+      <c r="Q37" s="58" t="n"/>
+      <c r="R37" s="58" t="n"/>
+      <c r="S37" s="58" t="n"/>
+      <c r="T37" s="53" t="n"/>
+      <c r="U37" s="58" t="n"/>
+      <c r="V37" s="53" t="n"/>
+      <c r="W37" s="53" t="n"/>
+      <c r="X37" s="58" t="n"/>
+      <c r="Y37" s="58" t="n"/>
+      <c r="Z37" s="58" t="n"/>
+      <c r="AA37" s="58" t="n"/>
+      <c r="AB37" s="58" t="n"/>
+      <c r="AC37" s="58" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="53" t="n"/>
-      <c r="B38" s="53" t="n"/>
-      <c r="C38" s="52" t="n"/>
+      <c r="B38" s="52" t="n"/>
+      <c r="C38" s="53" t="n"/>
       <c r="D38" s="53" t="n"/>
       <c r="E38" s="53" t="n"/>
-      <c r="F38" s="53" t="n"/>
-      <c r="G38" s="53" t="n"/>
-      <c r="H38" s="53" t="n"/>
+      <c r="F38" s="58" t="n"/>
+      <c r="G38" s="58" t="n"/>
+      <c r="H38" s="58" t="n"/>
+      <c r="I38" s="58" t="n"/>
+      <c r="J38" s="58" t="n"/>
+      <c r="K38" s="58" t="n"/>
+      <c r="L38" s="58" t="n"/>
+      <c r="M38" s="58" t="n"/>
+      <c r="N38" s="58" t="n"/>
+      <c r="O38" s="58" t="n"/>
+      <c r="P38" s="58" t="n"/>
+      <c r="Q38" s="58" t="n"/>
+      <c r="R38" s="58" t="n"/>
+      <c r="S38" s="58" t="n"/>
+      <c r="T38" s="53" t="n"/>
+      <c r="U38" s="58" t="n"/>
+      <c r="V38" s="53" t="n"/>
+      <c r="W38" s="53" t="n"/>
+      <c r="X38" s="58" t="n"/>
+      <c r="Y38" s="58" t="n"/>
+      <c r="Z38" s="58" t="n"/>
+      <c r="AA38" s="58" t="n"/>
+      <c r="AB38" s="58" t="n"/>
+      <c r="AC38" s="58" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="53" t="n"/>
-      <c r="B39" s="53" t="n"/>
-      <c r="C39" s="52" t="n"/>
+      <c r="B39" s="52" t="n"/>
+      <c r="C39" s="53" t="n"/>
       <c r="D39" s="53" t="n"/>
       <c r="E39" s="53" t="n"/>
-      <c r="F39" s="53" t="n"/>
-      <c r="G39" s="53" t="n"/>
-      <c r="H39" s="53" t="n"/>
+      <c r="F39" s="58" t="n"/>
+      <c r="G39" s="58" t="n"/>
+      <c r="H39" s="58" t="n"/>
+      <c r="I39" s="58" t="n"/>
+      <c r="J39" s="58" t="n"/>
+      <c r="K39" s="58" t="n"/>
+      <c r="L39" s="58" t="n"/>
+      <c r="M39" s="58" t="n"/>
+      <c r="N39" s="58" t="n"/>
+      <c r="O39" s="58" t="n"/>
+      <c r="P39" s="58" t="n"/>
+      <c r="Q39" s="58" t="n"/>
+      <c r="R39" s="58" t="n"/>
+      <c r="S39" s="58" t="n"/>
+      <c r="T39" s="53" t="n"/>
+      <c r="U39" s="58" t="n"/>
+      <c r="V39" s="53" t="n"/>
+      <c r="W39" s="53" t="n"/>
+      <c r="X39" s="58" t="n"/>
+      <c r="Y39" s="58" t="n"/>
+      <c r="Z39" s="58" t="n"/>
+      <c r="AA39" s="58" t="n"/>
+      <c r="AB39" s="58" t="n"/>
+      <c r="AC39" s="58" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="53" t="n"/>
-      <c r="B40" s="53" t="n"/>
-      <c r="C40" s="52" t="n"/>
+      <c r="B40" s="52" t="n"/>
+      <c r="C40" s="53" t="n"/>
       <c r="D40" s="53" t="n"/>
       <c r="E40" s="53" t="n"/>
-      <c r="F40" s="53" t="n"/>
-      <c r="G40" s="53" t="n"/>
-      <c r="H40" s="53" t="n"/>
+      <c r="F40" s="58" t="n"/>
+      <c r="G40" s="58" t="n"/>
+      <c r="H40" s="58" t="n"/>
+      <c r="I40" s="58" t="n"/>
+      <c r="J40" s="58" t="n"/>
+      <c r="K40" s="58" t="n"/>
+      <c r="L40" s="58" t="n"/>
+      <c r="M40" s="58" t="n"/>
+      <c r="N40" s="58" t="n"/>
+      <c r="O40" s="58" t="n"/>
+      <c r="P40" s="58" t="n"/>
+      <c r="Q40" s="58" t="n"/>
+      <c r="R40" s="58" t="n"/>
+      <c r="S40" s="58" t="n"/>
+      <c r="T40" s="53" t="n"/>
+      <c r="U40" s="58" t="n"/>
+      <c r="V40" s="53" t="n"/>
+      <c r="W40" s="53" t="n"/>
+      <c r="X40" s="58" t="n"/>
+      <c r="Y40" s="58" t="n"/>
+      <c r="Z40" s="58" t="n"/>
+      <c r="AA40" s="58" t="n"/>
+      <c r="AB40" s="58" t="n"/>
+      <c r="AC40" s="58" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="53" t="n"/>
-      <c r="B41" s="53" t="n"/>
-      <c r="C41" s="52" t="n"/>
+      <c r="B41" s="52" t="n"/>
+      <c r="C41" s="53" t="n"/>
       <c r="D41" s="53" t="n"/>
       <c r="E41" s="53" t="n"/>
-      <c r="F41" s="53" t="n"/>
-      <c r="G41" s="53" t="n"/>
-      <c r="H41" s="53" t="n"/>
+      <c r="F41" s="58" t="n"/>
+      <c r="G41" s="58" t="n"/>
+      <c r="H41" s="58" t="n"/>
+      <c r="I41" s="58" t="n"/>
+      <c r="J41" s="58" t="n"/>
+      <c r="K41" s="58" t="n"/>
+      <c r="L41" s="58" t="n"/>
+      <c r="M41" s="58" t="n"/>
+      <c r="N41" s="58" t="n"/>
+      <c r="O41" s="58" t="n"/>
+      <c r="P41" s="58" t="n"/>
+      <c r="Q41" s="58" t="n"/>
+      <c r="R41" s="58" t="n"/>
+      <c r="S41" s="58" t="n"/>
+      <c r="T41" s="53" t="n"/>
+      <c r="U41" s="58" t="n"/>
+      <c r="V41" s="53" t="n"/>
+      <c r="W41" s="53" t="n"/>
+      <c r="X41" s="58" t="n"/>
+      <c r="Y41" s="58" t="n"/>
+      <c r="Z41" s="58" t="n"/>
+      <c r="AA41" s="58" t="n"/>
+      <c r="AB41" s="58" t="n"/>
+      <c r="AC41" s="58" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="53" t="n"/>
-      <c r="B42" s="53" t="n"/>
-      <c r="C42" s="52" t="n"/>
+      <c r="B42" s="52" t="n"/>
+      <c r="C42" s="53" t="n"/>
       <c r="D42" s="53" t="n"/>
       <c r="E42" s="53" t="n"/>
-      <c r="F42" s="53" t="n"/>
-      <c r="G42" s="53" t="n"/>
-      <c r="H42" s="53" t="n"/>
+      <c r="F42" s="58" t="n"/>
+      <c r="G42" s="58" t="n"/>
+      <c r="H42" s="58" t="n"/>
+      <c r="I42" s="58" t="n"/>
+      <c r="J42" s="58" t="n"/>
+      <c r="K42" s="58" t="n"/>
+      <c r="L42" s="58" t="n"/>
+      <c r="M42" s="58" t="n"/>
+      <c r="N42" s="58" t="n"/>
+      <c r="O42" s="58" t="n"/>
+      <c r="P42" s="58" t="n"/>
+      <c r="Q42" s="58" t="n"/>
+      <c r="R42" s="58" t="n"/>
+      <c r="S42" s="58" t="n"/>
+      <c r="T42" s="53" t="n"/>
+      <c r="U42" s="58" t="n"/>
+      <c r="V42" s="53" t="n"/>
+      <c r="W42" s="53" t="n"/>
+      <c r="X42" s="58" t="n"/>
+      <c r="Y42" s="58" t="n"/>
+      <c r="Z42" s="58" t="n"/>
+      <c r="AA42" s="58" t="n"/>
+      <c r="AB42" s="58" t="n"/>
+      <c r="AC42" s="58" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="53" t="n"/>
-      <c r="B43" s="53" t="n"/>
-      <c r="C43" s="52" t="n"/>
+      <c r="B43" s="52" t="n"/>
+      <c r="C43" s="53" t="n"/>
       <c r="D43" s="53" t="n"/>
       <c r="E43" s="53" t="n"/>
-      <c r="F43" s="53" t="n"/>
-      <c r="G43" s="53" t="n"/>
-      <c r="H43" s="53" t="n"/>
+      <c r="F43" s="58" t="n"/>
+      <c r="G43" s="58" t="n"/>
+      <c r="H43" s="58" t="n"/>
+      <c r="I43" s="58" t="n"/>
+      <c r="J43" s="58" t="n"/>
+      <c r="K43" s="58" t="n"/>
+      <c r="L43" s="58" t="n"/>
+      <c r="M43" s="58" t="n"/>
+      <c r="N43" s="58" t="n"/>
+      <c r="O43" s="58" t="n"/>
+      <c r="P43" s="58" t="n"/>
+      <c r="Q43" s="58" t="n"/>
+      <c r="R43" s="58" t="n"/>
+      <c r="S43" s="58" t="n"/>
+      <c r="T43" s="53" t="n"/>
+      <c r="U43" s="58" t="n"/>
+      <c r="V43" s="53" t="n"/>
+      <c r="W43" s="53" t="n"/>
+      <c r="X43" s="58" t="n"/>
+      <c r="Y43" s="58" t="n"/>
+      <c r="Z43" s="58" t="n"/>
+      <c r="AA43" s="58" t="n"/>
+      <c r="AB43" s="58" t="n"/>
+      <c r="AC43" s="58" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="53" t="n"/>
-      <c r="B44" s="53" t="n"/>
-      <c r="C44" s="52" t="n"/>
+      <c r="B44" s="52" t="n"/>
+      <c r="C44" s="53" t="n"/>
       <c r="D44" s="53" t="n"/>
       <c r="E44" s="53" t="n"/>
-      <c r="F44" s="53" t="n"/>
-      <c r="G44" s="53" t="n"/>
-      <c r="H44" s="53" t="n"/>
+      <c r="F44" s="58" t="n"/>
+      <c r="G44" s="58" t="n"/>
+      <c r="H44" s="58" t="n"/>
+      <c r="I44" s="58" t="n"/>
+      <c r="J44" s="58" t="n"/>
+      <c r="K44" s="58" t="n"/>
+      <c r="L44" s="58" t="n"/>
+      <c r="M44" s="58" t="n"/>
+      <c r="N44" s="58" t="n"/>
+      <c r="O44" s="58" t="n"/>
+      <c r="P44" s="58" t="n"/>
+      <c r="Q44" s="58" t="n"/>
+      <c r="R44" s="58" t="n"/>
+      <c r="S44" s="58" t="n"/>
+      <c r="T44" s="53" t="n"/>
+      <c r="U44" s="58" t="n"/>
+      <c r="V44" s="53" t="n"/>
+      <c r="W44" s="53" t="n"/>
+      <c r="X44" s="58" t="n"/>
+      <c r="Y44" s="58" t="n"/>
+      <c r="Z44" s="58" t="n"/>
+      <c r="AA44" s="58" t="n"/>
+      <c r="AB44" s="58" t="n"/>
+      <c r="AC44" s="58" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="53" t="n"/>
-      <c r="B45" s="53" t="n"/>
-      <c r="C45" s="52" t="n"/>
+      <c r="B45" s="52" t="n"/>
+      <c r="C45" s="53" t="n"/>
       <c r="D45" s="53" t="n"/>
       <c r="E45" s="53" t="n"/>
-      <c r="F45" s="53" t="n"/>
-      <c r="G45" s="53" t="n"/>
-      <c r="H45" s="53" t="n"/>
+      <c r="F45" s="58" t="n"/>
+      <c r="G45" s="58" t="n"/>
+      <c r="H45" s="58" t="n"/>
+      <c r="I45" s="58" t="n"/>
+      <c r="J45" s="58" t="n"/>
+      <c r="K45" s="58" t="n"/>
+      <c r="L45" s="58" t="n"/>
+      <c r="M45" s="58" t="n"/>
+      <c r="N45" s="58" t="n"/>
+      <c r="O45" s="58" t="n"/>
+      <c r="P45" s="58" t="n"/>
+      <c r="Q45" s="58" t="n"/>
+      <c r="R45" s="58" t="n"/>
+      <c r="S45" s="58" t="n"/>
+      <c r="T45" s="53" t="n"/>
+      <c r="U45" s="58" t="n"/>
+      <c r="V45" s="53" t="n"/>
+      <c r="W45" s="53" t="n"/>
+      <c r="X45" s="58" t="n"/>
+      <c r="Y45" s="58" t="n"/>
+      <c r="Z45" s="58" t="n"/>
+      <c r="AA45" s="58" t="n"/>
+      <c r="AB45" s="58" t="n"/>
+      <c r="AC45" s="58" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="53" t="n"/>
-      <c r="B46" s="53" t="n"/>
-      <c r="C46" s="52" t="n"/>
+      <c r="B46" s="52" t="n"/>
+      <c r="C46" s="53" t="n"/>
       <c r="D46" s="53" t="n"/>
       <c r="E46" s="53" t="n"/>
-      <c r="F46" s="53" t="n"/>
-      <c r="G46" s="53" t="n"/>
-      <c r="H46" s="53" t="n"/>
+      <c r="F46" s="58" t="n"/>
+      <c r="G46" s="58" t="n"/>
+      <c r="H46" s="58" t="n"/>
+      <c r="I46" s="58" t="n"/>
+      <c r="J46" s="58" t="n"/>
+      <c r="K46" s="58" t="n"/>
+      <c r="L46" s="58" t="n"/>
+      <c r="M46" s="58" t="n"/>
+      <c r="N46" s="58" t="n"/>
+      <c r="O46" s="58" t="n"/>
+      <c r="P46" s="58" t="n"/>
+      <c r="Q46" s="58" t="n"/>
+      <c r="R46" s="58" t="n"/>
+      <c r="S46" s="58" t="n"/>
+      <c r="T46" s="53" t="n"/>
+      <c r="U46" s="58" t="n"/>
+      <c r="V46" s="53" t="n"/>
+      <c r="W46" s="53" t="n"/>
+      <c r="X46" s="58" t="n"/>
+      <c r="Y46" s="58" t="n"/>
+      <c r="Z46" s="58" t="n"/>
+      <c r="AA46" s="58" t="n"/>
+      <c r="AB46" s="58" t="n"/>
+      <c r="AC46" s="58" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="53" t="n"/>
-      <c r="B47" s="53" t="n"/>
-      <c r="C47" s="52" t="n"/>
+      <c r="B47" s="52" t="n"/>
+      <c r="C47" s="53" t="n"/>
       <c r="D47" s="53" t="n"/>
       <c r="E47" s="53" t="n"/>
-      <c r="F47" s="53" t="n"/>
-      <c r="G47" s="53" t="n"/>
-      <c r="H47" s="53" t="n"/>
+      <c r="F47" s="58" t="n"/>
+      <c r="G47" s="58" t="n"/>
+      <c r="H47" s="58" t="n"/>
+      <c r="I47" s="58" t="n"/>
+      <c r="J47" s="58" t="n"/>
+      <c r="K47" s="58" t="n"/>
+      <c r="L47" s="58" t="n"/>
+      <c r="M47" s="58" t="n"/>
+      <c r="N47" s="58" t="n"/>
+      <c r="O47" s="58" t="n"/>
+      <c r="P47" s="58" t="n"/>
+      <c r="Q47" s="58" t="n"/>
+      <c r="R47" s="58" t="n"/>
+      <c r="S47" s="58" t="n"/>
+      <c r="T47" s="53" t="n"/>
+      <c r="U47" s="58" t="n"/>
+      <c r="V47" s="53" t="n"/>
+      <c r="W47" s="53" t="n"/>
+      <c r="X47" s="58" t="n"/>
+      <c r="Y47" s="58" t="n"/>
+      <c r="Z47" s="58" t="n"/>
+      <c r="AA47" s="58" t="n"/>
+      <c r="AB47" s="58" t="n"/>
+      <c r="AC47" s="58" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="53" t="n"/>
-      <c r="B48" s="53" t="n"/>
-      <c r="C48" s="52" t="n"/>
+      <c r="B48" s="52" t="n"/>
+      <c r="C48" s="53" t="n"/>
       <c r="D48" s="53" t="n"/>
       <c r="E48" s="53" t="n"/>
-      <c r="F48" s="53" t="n"/>
-      <c r="G48" s="53" t="n"/>
-      <c r="H48" s="53" t="n"/>
+      <c r="F48" s="58" t="n"/>
+      <c r="G48" s="58" t="n"/>
+      <c r="H48" s="58" t="n"/>
+      <c r="I48" s="58" t="n"/>
+      <c r="J48" s="58" t="n"/>
+      <c r="K48" s="58" t="n"/>
+      <c r="L48" s="58" t="n"/>
+      <c r="M48" s="58" t="n"/>
+      <c r="N48" s="58" t="n"/>
+      <c r="O48" s="58" t="n"/>
+      <c r="P48" s="58" t="n"/>
+      <c r="Q48" s="58" t="n"/>
+      <c r="R48" s="58" t="n"/>
+      <c r="S48" s="58" t="n"/>
+      <c r="T48" s="53" t="n"/>
+      <c r="U48" s="58" t="n"/>
+      <c r="V48" s="53" t="n"/>
+      <c r="W48" s="53" t="n"/>
+      <c r="X48" s="58" t="n"/>
+      <c r="Y48" s="58" t="n"/>
+      <c r="Z48" s="58" t="n"/>
+      <c r="AA48" s="58" t="n"/>
+      <c r="AB48" s="58" t="n"/>
+      <c r="AC48" s="58" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="53" t="n"/>
-      <c r="B49" s="53" t="n"/>
-      <c r="C49" s="52" t="n"/>
+      <c r="B49" s="52" t="n"/>
+      <c r="C49" s="53" t="n"/>
       <c r="D49" s="53" t="n"/>
       <c r="E49" s="53" t="n"/>
-      <c r="F49" s="53" t="n"/>
-      <c r="G49" s="53" t="n"/>
-      <c r="H49" s="53" t="n"/>
+      <c r="F49" s="58" t="n"/>
+      <c r="G49" s="58" t="n"/>
+      <c r="H49" s="58" t="n"/>
+      <c r="I49" s="58" t="n"/>
+      <c r="J49" s="58" t="n"/>
+      <c r="K49" s="58" t="n"/>
+      <c r="L49" s="58" t="n"/>
+      <c r="M49" s="58" t="n"/>
+      <c r="N49" s="58" t="n"/>
+      <c r="O49" s="58" t="n"/>
+      <c r="P49" s="58" t="n"/>
+      <c r="Q49" s="58" t="n"/>
+      <c r="R49" s="58" t="n"/>
+      <c r="S49" s="58" t="n"/>
+      <c r="T49" s="53" t="n"/>
+      <c r="U49" s="58" t="n"/>
+      <c r="V49" s="53" t="n"/>
+      <c r="W49" s="53" t="n"/>
+      <c r="X49" s="58" t="n"/>
+      <c r="Y49" s="58" t="n"/>
+      <c r="Z49" s="58" t="n"/>
+      <c r="AA49" s="58" t="n"/>
+      <c r="AB49" s="58" t="n"/>
+      <c r="AC49" s="58" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="53" t="n"/>
-      <c r="B50" s="53" t="n"/>
-      <c r="C50" s="52" t="n"/>
+      <c r="B50" s="52" t="n"/>
+      <c r="C50" s="53" t="n"/>
       <c r="D50" s="53" t="n"/>
       <c r="E50" s="53" t="n"/>
-      <c r="F50" s="53" t="n"/>
-      <c r="G50" s="53" t="n"/>
-      <c r="H50" s="53" t="n"/>
+      <c r="F50" s="58" t="n"/>
+      <c r="G50" s="58" t="n"/>
+      <c r="H50" s="58" t="n"/>
+      <c r="I50" s="58" t="n"/>
+      <c r="J50" s="58" t="n"/>
+      <c r="K50" s="58" t="n"/>
+      <c r="L50" s="58" t="n"/>
+      <c r="M50" s="58" t="n"/>
+      <c r="N50" s="58" t="n"/>
+      <c r="O50" s="58" t="n"/>
+      <c r="P50" s="58" t="n"/>
+      <c r="Q50" s="58" t="n"/>
+      <c r="R50" s="58" t="n"/>
+      <c r="S50" s="58" t="n"/>
+      <c r="T50" s="53" t="n"/>
+      <c r="U50" s="58" t="n"/>
+      <c r="V50" s="53" t="n"/>
+      <c r="W50" s="53" t="n"/>
+      <c r="X50" s="58" t="n"/>
+      <c r="Y50" s="58" t="n"/>
+      <c r="Z50" s="58" t="n"/>
+      <c r="AA50" s="58" t="n"/>
+      <c r="AB50" s="58" t="n"/>
+      <c r="AC50" s="58" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="53" t="n"/>
-      <c r="B51" s="53" t="n"/>
-      <c r="C51" s="52" t="n"/>
+      <c r="B51" s="52" t="n"/>
+      <c r="C51" s="53" t="n"/>
       <c r="D51" s="53" t="n"/>
       <c r="E51" s="53" t="n"/>
-      <c r="F51" s="53" t="n"/>
-      <c r="G51" s="53" t="n"/>
-      <c r="H51" s="53" t="n"/>
+      <c r="F51" s="58" t="n"/>
+      <c r="G51" s="58" t="n"/>
+      <c r="H51" s="58" t="n"/>
+      <c r="I51" s="58" t="n"/>
+      <c r="J51" s="58" t="n"/>
+      <c r="K51" s="58" t="n"/>
+      <c r="L51" s="58" t="n"/>
+      <c r="M51" s="58" t="n"/>
+      <c r="N51" s="58" t="n"/>
+      <c r="O51" s="58" t="n"/>
+      <c r="P51" s="58" t="n"/>
+      <c r="Q51" s="58" t="n"/>
+      <c r="R51" s="58" t="n"/>
+      <c r="S51" s="58" t="n"/>
+      <c r="T51" s="53" t="n"/>
+      <c r="U51" s="58" t="n"/>
+      <c r="V51" s="53" t="n"/>
+      <c r="W51" s="53" t="n"/>
+      <c r="X51" s="58" t="n"/>
+      <c r="Y51" s="58" t="n"/>
+      <c r="Z51" s="58" t="n"/>
+      <c r="AA51" s="58" t="n"/>
+      <c r="AB51" s="58" t="n"/>
+      <c r="AC51" s="58" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="53" t="n"/>
-      <c r="B52" s="53" t="n"/>
-      <c r="C52" s="52" t="n"/>
+      <c r="B52" s="52" t="n"/>
+      <c r="C52" s="53" t="n"/>
       <c r="D52" s="53" t="n"/>
       <c r="E52" s="53" t="n"/>
-      <c r="F52" s="53" t="n"/>
-      <c r="G52" s="53" t="n"/>
-      <c r="H52" s="53" t="n"/>
+      <c r="F52" s="58" t="n"/>
+      <c r="G52" s="58" t="n"/>
+      <c r="H52" s="58" t="n"/>
+      <c r="I52" s="58" t="n"/>
+      <c r="J52" s="58" t="n"/>
+      <c r="K52" s="58" t="n"/>
+      <c r="L52" s="58" t="n"/>
+      <c r="M52" s="58" t="n"/>
+      <c r="N52" s="58" t="n"/>
+      <c r="O52" s="58" t="n"/>
+      <c r="P52" s="58" t="n"/>
+      <c r="Q52" s="58" t="n"/>
+      <c r="R52" s="58" t="n"/>
+      <c r="S52" s="58" t="n"/>
+      <c r="T52" s="53" t="n"/>
+      <c r="U52" s="58" t="n"/>
+      <c r="V52" s="53" t="n"/>
+      <c r="W52" s="53" t="n"/>
+      <c r="X52" s="58" t="n"/>
+      <c r="Y52" s="58" t="n"/>
+      <c r="Z52" s="58" t="n"/>
+      <c r="AA52" s="58" t="n"/>
+      <c r="AB52" s="58" t="n"/>
+      <c r="AC52" s="58" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="53" t="n"/>
-      <c r="B53" s="53" t="n"/>
-      <c r="C53" s="52" t="n"/>
+      <c r="B53" s="52" t="n"/>
+      <c r="C53" s="53" t="n"/>
       <c r="D53" s="53" t="n"/>
       <c r="E53" s="53" t="n"/>
-      <c r="F53" s="53" t="n"/>
-      <c r="G53" s="53" t="n"/>
-      <c r="H53" s="53" t="n"/>
+      <c r="F53" s="58" t="n"/>
+      <c r="G53" s="58" t="n"/>
+      <c r="H53" s="58" t="n"/>
+      <c r="I53" s="58" t="n"/>
+      <c r="J53" s="58" t="n"/>
+      <c r="K53" s="58" t="n"/>
+      <c r="L53" s="58" t="n"/>
+      <c r="M53" s="58" t="n"/>
+      <c r="N53" s="58" t="n"/>
+      <c r="O53" s="58" t="n"/>
+      <c r="P53" s="58" t="n"/>
+      <c r="Q53" s="58" t="n"/>
+      <c r="R53" s="58" t="n"/>
+      <c r="S53" s="58" t="n"/>
+      <c r="T53" s="53" t="n"/>
+      <c r="U53" s="58" t="n"/>
+      <c r="V53" s="53" t="n"/>
+      <c r="W53" s="53" t="n"/>
+      <c r="X53" s="58" t="n"/>
+      <c r="Y53" s="58" t="n"/>
+      <c r="Z53" s="58" t="n"/>
+      <c r="AA53" s="58" t="n"/>
+      <c r="AB53" s="58" t="n"/>
+      <c r="AC53" s="58" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="53" t="n"/>
-      <c r="B54" s="53" t="n"/>
-      <c r="C54" s="52" t="n"/>
+      <c r="B54" s="52" t="n"/>
+      <c r="C54" s="53" t="n"/>
       <c r="D54" s="53" t="n"/>
       <c r="E54" s="53" t="n"/>
-      <c r="F54" s="53" t="n"/>
-      <c r="G54" s="53" t="n"/>
-      <c r="H54" s="53" t="n"/>
+      <c r="F54" s="58" t="n"/>
+      <c r="G54" s="58" t="n"/>
+      <c r="H54" s="58" t="n"/>
+      <c r="I54" s="58" t="n"/>
+      <c r="J54" s="58" t="n"/>
+      <c r="K54" s="58" t="n"/>
+      <c r="L54" s="58" t="n"/>
+      <c r="M54" s="58" t="n"/>
+      <c r="N54" s="58" t="n"/>
+      <c r="O54" s="58" t="n"/>
+      <c r="P54" s="58" t="n"/>
+      <c r="Q54" s="58" t="n"/>
+      <c r="R54" s="58" t="n"/>
+      <c r="S54" s="58" t="n"/>
+      <c r="T54" s="53" t="n"/>
+      <c r="U54" s="58" t="n"/>
+      <c r="V54" s="53" t="n"/>
+      <c r="W54" s="53" t="n"/>
+      <c r="X54" s="58" t="n"/>
+      <c r="Y54" s="58" t="n"/>
+      <c r="Z54" s="58" t="n"/>
+      <c r="AA54" s="58" t="n"/>
+      <c r="AB54" s="58" t="n"/>
+      <c r="AC54" s="58" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="53" t="n"/>
-      <c r="B55" s="53" t="n"/>
-      <c r="C55" s="52" t="n"/>
+      <c r="B55" s="52" t="n"/>
+      <c r="C55" s="53" t="n"/>
       <c r="D55" s="53" t="n"/>
       <c r="E55" s="53" t="n"/>
-      <c r="F55" s="53" t="n"/>
-      <c r="G55" s="53" t="n"/>
-      <c r="H55" s="53" t="n"/>
+      <c r="F55" s="58" t="n"/>
+      <c r="G55" s="58" t="n"/>
+      <c r="H55" s="58" t="n"/>
+      <c r="I55" s="58" t="n"/>
+      <c r="J55" s="58" t="n"/>
+      <c r="K55" s="58" t="n"/>
+      <c r="L55" s="58" t="n"/>
+      <c r="M55" s="58" t="n"/>
+      <c r="N55" s="58" t="n"/>
+      <c r="O55" s="58" t="n"/>
+      <c r="P55" s="58" t="n"/>
+      <c r="Q55" s="58" t="n"/>
+      <c r="R55" s="58" t="n"/>
+      <c r="S55" s="58" t="n"/>
+      <c r="T55" s="53" t="n"/>
+      <c r="U55" s="58" t="n"/>
+      <c r="V55" s="53" t="n"/>
+      <c r="W55" s="53" t="n"/>
+      <c r="X55" s="58" t="n"/>
+      <c r="Y55" s="58" t="n"/>
+      <c r="Z55" s="58" t="n"/>
+      <c r="AA55" s="58" t="n"/>
+      <c r="AB55" s="58" t="n"/>
+      <c r="AC55" s="58" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="53" t="n"/>
-      <c r="B56" s="53" t="n"/>
-      <c r="C56" s="52" t="n"/>
+      <c r="B56" s="52" t="n"/>
+      <c r="C56" s="53" t="n"/>
       <c r="D56" s="53" t="n"/>
       <c r="E56" s="53" t="n"/>
-      <c r="F56" s="53" t="n"/>
-      <c r="G56" s="53" t="n"/>
-      <c r="H56" s="53" t="n"/>
+      <c r="F56" s="58" t="n"/>
+      <c r="G56" s="58" t="n"/>
+      <c r="H56" s="58" t="n"/>
+      <c r="I56" s="58" t="n"/>
+      <c r="J56" s="58" t="n"/>
+      <c r="K56" s="58" t="n"/>
+      <c r="L56" s="58" t="n"/>
+      <c r="M56" s="58" t="n"/>
+      <c r="N56" s="58" t="n"/>
+      <c r="O56" s="58" t="n"/>
+      <c r="P56" s="58" t="n"/>
+      <c r="Q56" s="58" t="n"/>
+      <c r="R56" s="58" t="n"/>
+      <c r="S56" s="58" t="n"/>
+      <c r="T56" s="53" t="n"/>
+      <c r="U56" s="58" t="n"/>
+      <c r="V56" s="53" t="n"/>
+      <c r="W56" s="53" t="n"/>
+      <c r="X56" s="58" t="n"/>
+      <c r="Y56" s="58" t="n"/>
+      <c r="Z56" s="58" t="n"/>
+      <c r="AA56" s="58" t="n"/>
+      <c r="AB56" s="58" t="n"/>
+      <c r="AC56" s="58" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="53" t="n"/>
-      <c r="B57" s="53" t="n"/>
-      <c r="C57" s="52" t="n"/>
+      <c r="B57" s="52" t="n"/>
+      <c r="C57" s="53" t="n"/>
       <c r="D57" s="53" t="n"/>
       <c r="E57" s="53" t="n"/>
-      <c r="F57" s="53" t="n"/>
-      <c r="G57" s="53" t="n"/>
-      <c r="H57" s="53" t="n"/>
+      <c r="F57" s="58" t="n"/>
+      <c r="G57" s="58" t="n"/>
+      <c r="H57" s="58" t="n"/>
+      <c r="I57" s="58" t="n"/>
+      <c r="J57" s="58" t="n"/>
+      <c r="K57" s="58" t="n"/>
+      <c r="L57" s="58" t="n"/>
+      <c r="M57" s="58" t="n"/>
+      <c r="N57" s="58" t="n"/>
+      <c r="O57" s="58" t="n"/>
+      <c r="P57" s="58" t="n"/>
+      <c r="Q57" s="58" t="n"/>
+      <c r="R57" s="58" t="n"/>
+      <c r="S57" s="58" t="n"/>
+      <c r="T57" s="53" t="n"/>
+      <c r="U57" s="58" t="n"/>
+      <c r="V57" s="53" t="n"/>
+      <c r="W57" s="53" t="n"/>
+      <c r="X57" s="58" t="n"/>
+      <c r="Y57" s="58" t="n"/>
+      <c r="Z57" s="58" t="n"/>
+      <c r="AA57" s="58" t="n"/>
+      <c r="AB57" s="58" t="n"/>
+      <c r="AC57" s="58" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="53" t="n"/>
-      <c r="B58" s="53" t="n"/>
-      <c r="C58" s="52" t="n"/>
+      <c r="B58" s="52" t="n"/>
+      <c r="C58" s="53" t="n"/>
       <c r="D58" s="53" t="n"/>
       <c r="E58" s="53" t="n"/>
-      <c r="F58" s="53" t="n"/>
-      <c r="G58" s="53" t="n"/>
-      <c r="H58" s="53" t="n"/>
+      <c r="F58" s="58" t="n"/>
+      <c r="G58" s="58" t="n"/>
+      <c r="H58" s="58" t="n"/>
+      <c r="I58" s="58" t="n"/>
+      <c r="J58" s="58" t="n"/>
+      <c r="K58" s="58" t="n"/>
+      <c r="L58" s="58" t="n"/>
+      <c r="M58" s="58" t="n"/>
+      <c r="N58" s="58" t="n"/>
+      <c r="O58" s="58" t="n"/>
+      <c r="P58" s="58" t="n"/>
+      <c r="Q58" s="58" t="n"/>
+      <c r="R58" s="58" t="n"/>
+      <c r="S58" s="58" t="n"/>
+      <c r="T58" s="53" t="n"/>
+      <c r="U58" s="58" t="n"/>
+      <c r="V58" s="53" t="n"/>
+      <c r="W58" s="53" t="n"/>
+      <c r="X58" s="58" t="n"/>
+      <c r="Y58" s="58" t="n"/>
+      <c r="Z58" s="58" t="n"/>
+      <c r="AA58" s="58" t="n"/>
+      <c r="AB58" s="58" t="n"/>
+      <c r="AC58" s="58" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="53" t="n"/>
-      <c r="B59" s="53" t="n"/>
-      <c r="C59" s="52" t="n"/>
+      <c r="B59" s="52" t="n"/>
+      <c r="C59" s="53" t="n"/>
       <c r="D59" s="53" t="n"/>
       <c r="E59" s="53" t="n"/>
-      <c r="F59" s="53" t="n"/>
-      <c r="G59" s="53" t="n"/>
-      <c r="H59" s="53" t="n"/>
+      <c r="F59" s="58" t="n"/>
+      <c r="G59" s="58" t="n"/>
+      <c r="H59" s="58" t="n"/>
+      <c r="I59" s="58" t="n"/>
+      <c r="J59" s="58" t="n"/>
+      <c r="K59" s="58" t="n"/>
+      <c r="L59" s="58" t="n"/>
+      <c r="M59" s="58" t="n"/>
+      <c r="N59" s="58" t="n"/>
+      <c r="O59" s="58" t="n"/>
+      <c r="P59" s="58" t="n"/>
+      <c r="Q59" s="58" t="n"/>
+      <c r="R59" s="58" t="n"/>
+      <c r="S59" s="58" t="n"/>
+      <c r="T59" s="53" t="n"/>
+      <c r="U59" s="58" t="n"/>
+      <c r="V59" s="53" t="n"/>
+      <c r="W59" s="53" t="n"/>
+      <c r="X59" s="58" t="n"/>
+      <c r="Y59" s="58" t="n"/>
+      <c r="Z59" s="58" t="n"/>
+      <c r="AA59" s="58" t="n"/>
+      <c r="AB59" s="58" t="n"/>
+      <c r="AC59" s="58" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="53" t="n"/>
-      <c r="B60" s="53" t="n"/>
-      <c r="C60" s="52" t="n"/>
+      <c r="B60" s="52" t="n"/>
+      <c r="C60" s="53" t="n"/>
       <c r="D60" s="53" t="n"/>
       <c r="E60" s="53" t="n"/>
-      <c r="F60" s="53" t="n"/>
-      <c r="G60" s="53" t="n"/>
-      <c r="H60" s="53" t="n"/>
+      <c r="F60" s="58" t="n"/>
+      <c r="G60" s="58" t="n"/>
+      <c r="H60" s="58" t="n"/>
+      <c r="I60" s="58" t="n"/>
+      <c r="J60" s="58" t="n"/>
+      <c r="K60" s="58" t="n"/>
+      <c r="L60" s="58" t="n"/>
+      <c r="M60" s="58" t="n"/>
+      <c r="N60" s="58" t="n"/>
+      <c r="O60" s="58" t="n"/>
+      <c r="P60" s="58" t="n"/>
+      <c r="Q60" s="58" t="n"/>
+      <c r="R60" s="58" t="n"/>
+      <c r="S60" s="58" t="n"/>
+      <c r="T60" s="53" t="n"/>
+      <c r="U60" s="58" t="n"/>
+      <c r="V60" s="53" t="n"/>
+      <c r="W60" s="53" t="n"/>
+      <c r="X60" s="58" t="n"/>
+      <c r="Y60" s="58" t="n"/>
+      <c r="Z60" s="58" t="n"/>
+      <c r="AA60" s="58" t="n"/>
+      <c r="AB60" s="58" t="n"/>
+      <c r="AC60" s="58" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="53" t="n"/>
-      <c r="B61" s="53" t="n"/>
-      <c r="C61" s="52" t="n"/>
+      <c r="B61" s="52" t="n"/>
+      <c r="C61" s="53" t="n"/>
       <c r="D61" s="53" t="n"/>
       <c r="E61" s="53" t="n"/>
-      <c r="F61" s="53" t="n"/>
-      <c r="G61" s="53" t="n"/>
-      <c r="H61" s="53" t="n"/>
+      <c r="F61" s="58" t="n"/>
+      <c r="G61" s="58" t="n"/>
+      <c r="H61" s="58" t="n"/>
+      <c r="I61" s="58" t="n"/>
+      <c r="J61" s="58" t="n"/>
+      <c r="K61" s="58" t="n"/>
+      <c r="L61" s="58" t="n"/>
+      <c r="M61" s="58" t="n"/>
+      <c r="N61" s="58" t="n"/>
+      <c r="O61" s="58" t="n"/>
+      <c r="P61" s="58" t="n"/>
+      <c r="Q61" s="58" t="n"/>
+      <c r="R61" s="58" t="n"/>
+      <c r="S61" s="58" t="n"/>
+      <c r="T61" s="53" t="n"/>
+      <c r="U61" s="58" t="n"/>
+      <c r="V61" s="53" t="n"/>
+      <c r="W61" s="53" t="n"/>
+      <c r="X61" s="58" t="n"/>
+      <c r="Y61" s="58" t="n"/>
+      <c r="Z61" s="58" t="n"/>
+      <c r="AA61" s="58" t="n"/>
+      <c r="AB61" s="58" t="n"/>
+      <c r="AC61" s="58" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="53" t="n"/>
-      <c r="B62" s="53" t="n"/>
-      <c r="C62" s="52" t="n"/>
+      <c r="B62" s="52" t="n"/>
+      <c r="C62" s="53" t="n"/>
       <c r="D62" s="53" t="n"/>
       <c r="E62" s="53" t="n"/>
-      <c r="F62" s="53" t="n"/>
-      <c r="G62" s="53" t="n"/>
-      <c r="H62" s="53" t="n"/>
+      <c r="F62" s="58" t="n"/>
+      <c r="G62" s="58" t="n"/>
+      <c r="H62" s="58" t="n"/>
+      <c r="I62" s="58" t="n"/>
+      <c r="J62" s="58" t="n"/>
+      <c r="K62" s="58" t="n"/>
+      <c r="L62" s="58" t="n"/>
+      <c r="M62" s="58" t="n"/>
+      <c r="N62" s="58" t="n"/>
+      <c r="O62" s="58" t="n"/>
+      <c r="P62" s="58" t="n"/>
+      <c r="Q62" s="58" t="n"/>
+      <c r="R62" s="58" t="n"/>
+      <c r="S62" s="58" t="n"/>
+      <c r="T62" s="53" t="n"/>
+      <c r="U62" s="58" t="n"/>
+      <c r="V62" s="53" t="n"/>
+      <c r="W62" s="53" t="n"/>
+      <c r="X62" s="58" t="n"/>
+      <c r="Y62" s="58" t="n"/>
+      <c r="Z62" s="58" t="n"/>
+      <c r="AA62" s="58" t="n"/>
+      <c r="AB62" s="58" t="n"/>
+      <c r="AC62" s="58" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="53" t="n"/>
-      <c r="B63" s="53" t="n"/>
-      <c r="C63" s="52" t="n"/>
+      <c r="B63" s="52" t="n"/>
+      <c r="C63" s="53" t="n"/>
       <c r="D63" s="53" t="n"/>
       <c r="E63" s="53" t="n"/>
-      <c r="F63" s="53" t="n"/>
-      <c r="G63" s="53" t="n"/>
-      <c r="H63" s="53" t="n"/>
+      <c r="F63" s="58" t="n"/>
+      <c r="G63" s="58" t="n"/>
+      <c r="H63" s="58" t="n"/>
+      <c r="I63" s="58" t="n"/>
+      <c r="J63" s="58" t="n"/>
+      <c r="K63" s="58" t="n"/>
+      <c r="L63" s="58" t="n"/>
+      <c r="M63" s="58" t="n"/>
+      <c r="N63" s="58" t="n"/>
+      <c r="O63" s="58" t="n"/>
+      <c r="P63" s="58" t="n"/>
+      <c r="Q63" s="58" t="n"/>
+      <c r="R63" s="58" t="n"/>
+      <c r="S63" s="58" t="n"/>
+      <c r="T63" s="53" t="n"/>
+      <c r="U63" s="58" t="n"/>
+      <c r="V63" s="53" t="n"/>
+      <c r="W63" s="53" t="n"/>
+      <c r="X63" s="58" t="n"/>
+      <c r="Y63" s="58" t="n"/>
+      <c r="Z63" s="58" t="n"/>
+      <c r="AA63" s="58" t="n"/>
+      <c r="AB63" s="58" t="n"/>
+      <c r="AC63" s="58" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="53" t="n"/>
-      <c r="B64" s="53" t="n"/>
-      <c r="C64" s="52" t="n"/>
+      <c r="B64" s="52" t="n"/>
+      <c r="C64" s="53" t="n"/>
       <c r="D64" s="53" t="n"/>
       <c r="E64" s="53" t="n"/>
-      <c r="F64" s="53" t="n"/>
-      <c r="G64" s="53" t="n"/>
-      <c r="H64" s="53" t="n"/>
+      <c r="F64" s="58" t="n"/>
+      <c r="G64" s="58" t="n"/>
+      <c r="H64" s="58" t="n"/>
+      <c r="I64" s="58" t="n"/>
+      <c r="J64" s="58" t="n"/>
+      <c r="K64" s="58" t="n"/>
+      <c r="L64" s="58" t="n"/>
+      <c r="M64" s="58" t="n"/>
+      <c r="N64" s="58" t="n"/>
+      <c r="O64" s="58" t="n"/>
+      <c r="P64" s="58" t="n"/>
+      <c r="Q64" s="58" t="n"/>
+      <c r="R64" s="58" t="n"/>
+      <c r="S64" s="58" t="n"/>
+      <c r="T64" s="53" t="n"/>
+      <c r="U64" s="58" t="n"/>
+      <c r="V64" s="53" t="n"/>
+      <c r="W64" s="53" t="n"/>
+      <c r="X64" s="58" t="n"/>
+      <c r="Y64" s="58" t="n"/>
+      <c r="Z64" s="58" t="n"/>
+      <c r="AA64" s="58" t="n"/>
+      <c r="AB64" s="58" t="n"/>
+      <c r="AC64" s="58" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="53" t="n"/>
-      <c r="B65" s="53" t="n"/>
-      <c r="C65" s="52" t="n"/>
+      <c r="B65" s="52" t="n"/>
+      <c r="C65" s="53" t="n"/>
       <c r="D65" s="53" t="n"/>
       <c r="E65" s="53" t="n"/>
-      <c r="F65" s="53" t="n"/>
-      <c r="G65" s="53" t="n"/>
-      <c r="H65" s="53" t="n"/>
+      <c r="F65" s="58" t="n"/>
+      <c r="G65" s="58" t="n"/>
+      <c r="H65" s="58" t="n"/>
+      <c r="I65" s="58" t="n"/>
+      <c r="J65" s="58" t="n"/>
+      <c r="K65" s="58" t="n"/>
+      <c r="L65" s="58" t="n"/>
+      <c r="M65" s="58" t="n"/>
+      <c r="N65" s="58" t="n"/>
+      <c r="O65" s="58" t="n"/>
+      <c r="P65" s="58" t="n"/>
+      <c r="Q65" s="58" t="n"/>
+      <c r="R65" s="58" t="n"/>
+      <c r="S65" s="58" t="n"/>
+      <c r="T65" s="53" t="n"/>
+      <c r="U65" s="58" t="n"/>
+      <c r="V65" s="53" t="n"/>
+      <c r="W65" s="53" t="n"/>
+      <c r="X65" s="58" t="n"/>
+      <c r="Y65" s="58" t="n"/>
+      <c r="Z65" s="58" t="n"/>
+      <c r="AA65" s="58" t="n"/>
+      <c r="AB65" s="58" t="n"/>
+      <c r="AC65" s="58" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4867,7 +6491,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="58" t="inlineStr">
+      <c r="A1" s="59" t="inlineStr">
         <is>
           <t>Type de colisage</t>
         </is>

</xml_diff>

<commit_message>
BL : recherche série nombre/texte, onglet catalogue masqué
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XPwnZBmWUGhvYebrP3X3Z2
</commit_message>
<xml_diff>
--- a/bl_2027/BL_Enedril_2027.xlsx
+++ b/bl_2027/BL_Enedril_2027.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 Bon de livraison" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 Import devis" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 Catalogue outils" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 Catalogue outils" sheetId="3" state="hidden" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listes" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
@@ -1191,7 +1191,7 @@
         <v/>
       </c>
       <c r="L15" s="13">
-        <f>IF(OR(J15=0,K15=1,B15=""),0,IFERROR(MATCH(B15,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J15=0,K15=1,B15=""),0,IFERROR(MATCH(B15,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B15,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B15),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M15" s="20">
@@ -1250,7 +1250,7 @@
         <v/>
       </c>
       <c r="L16" s="13">
-        <f>IF(OR(J16=0,K16=1,B16=""),0,IFERROR(MATCH(B16,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J16=0,K16=1,B16=""),0,IFERROR(MATCH(B16,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B16,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B16),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M16" s="20">
@@ -1309,7 +1309,7 @@
         <v/>
       </c>
       <c r="L17" s="13">
-        <f>IF(OR(J17=0,K17=1,B17=""),0,IFERROR(MATCH(B17,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J17=0,K17=1,B17=""),0,IFERROR(MATCH(B17,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B17,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B17),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M17" s="20">
@@ -1368,7 +1368,7 @@
         <v/>
       </c>
       <c r="L18" s="13">
-        <f>IF(OR(J18=0,K18=1,B18=""),0,IFERROR(MATCH(B18,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J18=0,K18=1,B18=""),0,IFERROR(MATCH(B18,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B18,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B18),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M18" s="20">
@@ -1427,7 +1427,7 @@
         <v/>
       </c>
       <c r="L19" s="13">
-        <f>IF(OR(J19=0,K19=1,B19=""),0,IFERROR(MATCH(B19,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J19=0,K19=1,B19=""),0,IFERROR(MATCH(B19,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B19,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B19),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M19" s="20">
@@ -1486,7 +1486,7 @@
         <v/>
       </c>
       <c r="L20" s="13">
-        <f>IF(OR(J20=0,K20=1,B20=""),0,IFERROR(MATCH(B20,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J20=0,K20=1,B20=""),0,IFERROR(MATCH(B20,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B20,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B20),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M20" s="20">
@@ -1545,7 +1545,7 @@
         <v/>
       </c>
       <c r="L21" s="13">
-        <f>IF(OR(J21=0,K21=1,B21=""),0,IFERROR(MATCH(B21,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J21=0,K21=1,B21=""),0,IFERROR(MATCH(B21,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B21,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B21),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M21" s="20">
@@ -1604,7 +1604,7 @@
         <v/>
       </c>
       <c r="L22" s="13">
-        <f>IF(OR(J22=0,K22=1,B22=""),0,IFERROR(MATCH(B22,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J22=0,K22=1,B22=""),0,IFERROR(MATCH(B22,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B22,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B22),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M22" s="20">
@@ -1663,7 +1663,7 @@
         <v/>
       </c>
       <c r="L23" s="13">
-        <f>IF(OR(J23=0,K23=1,B23=""),0,IFERROR(MATCH(B23,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J23=0,K23=1,B23=""),0,IFERROR(MATCH(B23,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B23,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B23),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M23" s="20">
@@ -1722,7 +1722,7 @@
         <v/>
       </c>
       <c r="L24" s="13">
-        <f>IF(OR(J24=0,K24=1,B24=""),0,IFERROR(MATCH(B24,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J24=0,K24=1,B24=""),0,IFERROR(MATCH(B24,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B24,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B24),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M24" s="20">
@@ -1781,7 +1781,7 @@
         <v/>
       </c>
       <c r="L25" s="13">
-        <f>IF(OR(J25=0,K25=1,B25=""),0,IFERROR(MATCH(B25,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J25=0,K25=1,B25=""),0,IFERROR(MATCH(B25,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B25,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B25),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M25" s="20">
@@ -1840,7 +1840,7 @@
         <v/>
       </c>
       <c r="L26" s="13">
-        <f>IF(OR(J26=0,K26=1,B26=""),0,IFERROR(MATCH(B26,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J26=0,K26=1,B26=""),0,IFERROR(MATCH(B26,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B26,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B26),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M26" s="20">
@@ -1899,7 +1899,7 @@
         <v/>
       </c>
       <c r="L27" s="13">
-        <f>IF(OR(J27=0,K27=1,B27=""),0,IFERROR(MATCH(B27,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J27=0,K27=1,B27=""),0,IFERROR(MATCH(B27,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B27,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B27),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M27" s="20">
@@ -1958,7 +1958,7 @@
         <v/>
       </c>
       <c r="L28" s="13">
-        <f>IF(OR(J28=0,K28=1,B28=""),0,IFERROR(MATCH(B28,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J28=0,K28=1,B28=""),0,IFERROR(MATCH(B28,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B28,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B28),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M28" s="20">
@@ -2017,7 +2017,7 @@
         <v/>
       </c>
       <c r="L29" s="13">
-        <f>IF(OR(J29=0,K29=1,B29=""),0,IFERROR(MATCH(B29,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J29=0,K29=1,B29=""),0,IFERROR(MATCH(B29,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B29,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B29),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M29" s="20">
@@ -2076,7 +2076,7 @@
         <v/>
       </c>
       <c r="L30" s="13">
-        <f>IF(OR(J30=0,K30=1,B30=""),0,IFERROR(MATCH(B30,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J30=0,K30=1,B30=""),0,IFERROR(MATCH(B30,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B30,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B30),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M30" s="20">
@@ -2135,7 +2135,7 @@
         <v/>
       </c>
       <c r="L31" s="13">
-        <f>IF(OR(J31=0,K31=1,B31=""),0,IFERROR(MATCH(B31,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J31=0,K31=1,B31=""),0,IFERROR(MATCH(B31,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B31,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B31),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M31" s="20">
@@ -2194,7 +2194,7 @@
         <v/>
       </c>
       <c r="L32" s="13">
-        <f>IF(OR(J32=0,K32=1,B32=""),0,IFERROR(MATCH(B32,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J32=0,K32=1,B32=""),0,IFERROR(MATCH(B32,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B32,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B32),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M32" s="20">
@@ -2253,7 +2253,7 @@
         <v/>
       </c>
       <c r="L33" s="13">
-        <f>IF(OR(J33=0,K33=1,B33=""),0,IFERROR(MATCH(B33,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J33=0,K33=1,B33=""),0,IFERROR(MATCH(B33,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B33,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B33),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M33" s="20">
@@ -2312,7 +2312,7 @@
         <v/>
       </c>
       <c r="L34" s="13">
-        <f>IF(OR(J34=0,K34=1,B34=""),0,IFERROR(MATCH(B34,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J34=0,K34=1,B34=""),0,IFERROR(MATCH(B34,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B34,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B34),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M34" s="20">
@@ -2371,7 +2371,7 @@
         <v/>
       </c>
       <c r="L35" s="13">
-        <f>IF(OR(J35=0,K35=1,B35=""),0,IFERROR(MATCH(B35,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J35=0,K35=1,B35=""),0,IFERROR(MATCH(B35,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B35,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B35),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M35" s="20">
@@ -2430,7 +2430,7 @@
         <v/>
       </c>
       <c r="L36" s="13">
-        <f>IF(OR(J36=0,K36=1,B36=""),0,IFERROR(MATCH(B36,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J36=0,K36=1,B36=""),0,IFERROR(MATCH(B36,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B36,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B36),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M36" s="20">
@@ -2489,7 +2489,7 @@
         <v/>
       </c>
       <c r="L37" s="13">
-        <f>IF(OR(J37=0,K37=1,B37=""),0,IFERROR(MATCH(B37,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J37=0,K37=1,B37=""),0,IFERROR(MATCH(B37,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B37,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B37),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M37" s="20">
@@ -2548,7 +2548,7 @@
         <v/>
       </c>
       <c r="L38" s="13">
-        <f>IF(OR(J38=0,K38=1,B38=""),0,IFERROR(MATCH(B38,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J38=0,K38=1,B38=""),0,IFERROR(MATCH(B38,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B38,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B38),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M38" s="20">
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="L39" s="13">
-        <f>IF(OR(J39=0,K39=1,B39=""),0,IFERROR(MATCH(B39,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J39=0,K39=1,B39=""),0,IFERROR(MATCH(B39,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B39,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B39),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M39" s="20">
@@ -2666,7 +2666,7 @@
         <v/>
       </c>
       <c r="L40" s="13">
-        <f>IF(OR(J40=0,K40=1,B40=""),0,IFERROR(MATCH(B40,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J40=0,K40=1,B40=""),0,IFERROR(MATCH(B40,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B40,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B40),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M40" s="20">
@@ -2725,7 +2725,7 @@
         <v/>
       </c>
       <c r="L41" s="13">
-        <f>IF(OR(J41=0,K41=1,B41=""),0,IFERROR(MATCH(B41,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J41=0,K41=1,B41=""),0,IFERROR(MATCH(B41,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B41,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B41),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M41" s="20">
@@ -2784,7 +2784,7 @@
         <v/>
       </c>
       <c r="L42" s="13">
-        <f>IF(OR(J42=0,K42=1,B42=""),0,IFERROR(MATCH(B42,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J42=0,K42=1,B42=""),0,IFERROR(MATCH(B42,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B42,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B42),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M42" s="20">
@@ -2843,7 +2843,7 @@
         <v/>
       </c>
       <c r="L43" s="13">
-        <f>IF(OR(J43=0,K43=1,B43=""),0,IFERROR(MATCH(B43,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J43=0,K43=1,B43=""),0,IFERROR(MATCH(B43,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B43,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B43),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M43" s="20">
@@ -2902,7 +2902,7 @@
         <v/>
       </c>
       <c r="L44" s="13">
-        <f>IF(OR(J44=0,K44=1,B44=""),0,IFERROR(MATCH(B44,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J44=0,K44=1,B44=""),0,IFERROR(MATCH(B44,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B44,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B44),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M44" s="20">
@@ -2961,7 +2961,7 @@
         <v/>
       </c>
       <c r="L45" s="13">
-        <f>IF(OR(J45=0,K45=1,B45=""),0,IFERROR(MATCH(B45,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J45=0,K45=1,B45=""),0,IFERROR(MATCH(B45,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B45,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B45),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M45" s="20">
@@ -3020,7 +3020,7 @@
         <v/>
       </c>
       <c r="L46" s="13">
-        <f>IF(OR(J46=0,K46=1,B46=""),0,IFERROR(MATCH(B46,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J46=0,K46=1,B46=""),0,IFERROR(MATCH(B46,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B46,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B46),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M46" s="20">
@@ -3079,7 +3079,7 @@
         <v/>
       </c>
       <c r="L47" s="13">
-        <f>IF(OR(J47=0,K47=1,B47=""),0,IFERROR(MATCH(B47,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J47=0,K47=1,B47=""),0,IFERROR(MATCH(B47,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B47,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B47),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M47" s="20">
@@ -3138,7 +3138,7 @@
         <v/>
       </c>
       <c r="L48" s="13">
-        <f>IF(OR(J48=0,K48=1,B48=""),0,IFERROR(MATCH(B48,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J48=0,K48=1,B48=""),0,IFERROR(MATCH(B48,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B48,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B48),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M48" s="20">
@@ -3197,7 +3197,7 @@
         <v/>
       </c>
       <c r="L49" s="13">
-        <f>IF(OR(J49=0,K49=1,B49=""),0,IFERROR(MATCH(B49,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J49=0,K49=1,B49=""),0,IFERROR(MATCH(B49,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B49,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B49),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M49" s="20">
@@ -3256,7 +3256,7 @@
         <v/>
       </c>
       <c r="L50" s="13">
-        <f>IF(OR(J50=0,K50=1,B50=""),0,IFERROR(MATCH(B50,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J50=0,K50=1,B50=""),0,IFERROR(MATCH(B50,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B50,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B50),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M50" s="20">
@@ -3315,7 +3315,7 @@
         <v/>
       </c>
       <c r="L51" s="13">
-        <f>IF(OR(J51=0,K51=1,B51=""),0,IFERROR(MATCH(B51,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J51=0,K51=1,B51=""),0,IFERROR(MATCH(B51,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B51,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B51),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M51" s="20">
@@ -3374,7 +3374,7 @@
         <v/>
       </c>
       <c r="L52" s="13">
-        <f>IF(OR(J52=0,K52=1,B52=""),0,IFERROR(MATCH(B52,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J52=0,K52=1,B52=""),0,IFERROR(MATCH(B52,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B52,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B52),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M52" s="20">
@@ -3433,7 +3433,7 @@
         <v/>
       </c>
       <c r="L53" s="13">
-        <f>IF(OR(J53=0,K53=1,B53=""),0,IFERROR(MATCH(B53,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J53=0,K53=1,B53=""),0,IFERROR(MATCH(B53,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B53,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B53),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M53" s="20">
@@ -3492,7 +3492,7 @@
         <v/>
       </c>
       <c r="L54" s="13">
-        <f>IF(OR(J54=0,K54=1,B54=""),0,IFERROR(MATCH(B54,'3 Catalogue outils'!$A$6:$A$5005,0),0))</f>
+        <f>IF(OR(J54=0,K54=1,B54=""),0,IFERROR(MATCH(B54,'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(TEXT(B54,"0"),'3 Catalogue outils'!$A$6:$A$5005,0),IFERROR(MATCH(VALUE(B54),'3 Catalogue outils'!$A$6:$A$5005,0),0))))</f>
         <v/>
       </c>
       <c r="M54" s="20">

</xml_diff>